<commit_message>
Fix AC#1/AC#2 data extraction with Sheet1 fallback
</commit_message>
<xml_diff>
--- a/Dashboard_Template_30_Slides_Final.xlsx
+++ b/Dashboard_Template_30_Slides_Final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\0_Dashboad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{641B5EB6-6245-4FEC-8D6C-32BFFC1B98E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C90AA0E-ED4E-4E43-ADFD-D7DE25D44F8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="791" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="791" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Part 1 - Overview" sheetId="1" r:id="rId1"/>
@@ -4599,7 +4599,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.75" bestFit="1" customWidth="1"/>
@@ -4608,7 +4608,7 @@
     <col min="5" max="5" width="77.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4625,7 +4625,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -4642,7 +4642,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -4660,7 +4660,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -4678,7 +4678,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -4695,7 +4695,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -4712,7 +4712,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -4729,7 +4729,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>28</v>
       </c>
@@ -4757,9 +4757,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4776,7 +4776,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>35</v>
       </c>
@@ -4793,7 +4793,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>39</v>
       </c>
@@ -4811,7 +4811,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -4829,7 +4829,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>44</v>
       </c>
@@ -4847,7 +4847,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>44</v>
       </c>
@@ -4865,7 +4865,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>49</v>
       </c>
@@ -4883,7 +4883,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>53</v>
       </c>
@@ -4901,7 +4901,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>56</v>
       </c>
@@ -4930,9 +4930,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4955,7 +4955,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>62</v>
       </c>
@@ -4978,7 +4978,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>62</v>
       </c>
@@ -5001,7 +5001,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>67</v>
       </c>
@@ -5025,7 +5025,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>71</v>
       </c>
@@ -5049,7 +5049,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>75</v>
       </c>
@@ -5073,7 +5073,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>79</v>
       </c>
@@ -5096,7 +5096,7 @@
         <v>9.9166666666666661</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>82</v>
       </c>
@@ -5119,7 +5119,7 @@
         <v>13.064935064935066</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>85</v>
       </c>
@@ -5150,9 +5150,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G36"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="39.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5169,7 +5178,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>91</v>
       </c>
@@ -5187,7 +5196,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>95</v>
       </c>
@@ -5205,7 +5214,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>95</v>
       </c>
@@ -5223,7 +5232,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>101</v>
       </c>
@@ -5241,7 +5250,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>105</v>
       </c>
@@ -5259,7 +5268,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>105</v>
       </c>
@@ -5277,7 +5286,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>111</v>
       </c>
@@ -5294,7 +5303,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>111</v>
       </c>
@@ -5311,7 +5320,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>111</v>
       </c>
@@ -5328,7 +5337,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>111</v>
       </c>
@@ -5345,7 +5354,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>111</v>
       </c>
@@ -5363,7 +5372,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>111</v>
       </c>
@@ -5373,15 +5382,15 @@
       <c r="C13" t="s">
         <v>123</v>
       </c>
-      <c r="D13" t="e">
-        <f>GETPIVOTDATA("REMAIN",Sheet1!$Q$5,"ACTION PLAN","Acctance Plan AC#1 WK27","HANDLE","HUAWEI","Years (SO DATE)",2023)</f>
-        <v>#REF!</v>
+      <c r="D13">
+        <f>Sheet1!T20</f>
+        <v>10369.500000000002</v>
       </c>
       <c r="E13" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>111</v>
       </c>
@@ -5398,7 +5407,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>111</v>
       </c>
@@ -5408,15 +5417,15 @@
       <c r="C15" t="s">
         <v>123</v>
       </c>
-      <c r="D15" t="e">
-        <f>GETPIVOTDATA("REMAIN",Sheet1!$Q$5,"ACTION PLAN","Acctance Plan AC#1 WK27","HANDLE","HUAWEI","Years (SO DATE)",2025)</f>
-        <v>#REF!</v>
+      <c r="D15">
+        <f>Sheet1!T21</f>
+        <v>13164.900000000001</v>
       </c>
       <c r="E15" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>111</v>
       </c>
@@ -5426,15 +5435,15 @@
       <c r="C16" t="s">
         <v>123</v>
       </c>
-      <c r="D16" t="e">
-        <f>GETPIVOTDATA("REMAIN",Sheet1!$Q$5,"ACTION PLAN","Acctance Plan AC#1 WK27","HANDLE","HUAWEI","Years (SO DATE)",2026)</f>
-        <v>#REF!</v>
+      <c r="D16">
+        <f>Sheet1!T22</f>
+        <v>41220</v>
       </c>
       <c r="E16" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>111</v>
       </c>
@@ -5444,15 +5453,15 @@
       <c r="C17" t="s">
         <v>123</v>
       </c>
-      <c r="D17" t="e">
+      <c r="D17">
         <f>SUM(D13:D16)</f>
-        <v>#REF!</v>
+        <v>64754.400000000001</v>
       </c>
       <c r="E17" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>133</v>
       </c>
@@ -5462,15 +5471,15 @@
       <c r="C18" t="s">
         <v>135</v>
       </c>
-      <c r="D18" t="e">
-        <f>GETPIVOTDATA("REMAIN",Sheet1!$Q$5,"ACTION PLAN","ACTION PLAN AC#2 WK27","HANDLE","HUAWEI","Years (SO DATE)",2023)</f>
-        <v>#REF!</v>
+      <c r="D18">
+        <f>Sheet1!T10</f>
+        <v>43613.1</v>
       </c>
       <c r="E18" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>133</v>
       </c>
@@ -5480,15 +5489,15 @@
       <c r="C19" t="s">
         <v>135</v>
       </c>
-      <c r="D19" t="e">
-        <f>GETPIVOTDATA("REMAIN",Sheet1!$Q$5,"ACTION PLAN","ACTION PLAN AC#2 WK27","HANDLE","HUAWEI","Years (SO DATE)",2024)</f>
-        <v>#REF!</v>
+      <c r="D19">
+        <f>Sheet1!T11</f>
+        <v>12891.900000000001</v>
       </c>
       <c r="E19" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>133</v>
       </c>
@@ -5498,15 +5507,15 @@
       <c r="C20" t="s">
         <v>135</v>
       </c>
-      <c r="D20" t="e">
-        <f>GETPIVOTDATA("REMAIN",Sheet1!$Q$5,"ACTION PLAN","ACTION PLAN AC#2 WK27","HANDLE","HUAWEI","Years (SO DATE)",2025)</f>
-        <v>#REF!</v>
+      <c r="D20">
+        <f>Sheet1!T12</f>
+        <v>43148.100000000013</v>
       </c>
       <c r="E20" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>133</v>
       </c>
@@ -5516,15 +5525,15 @@
       <c r="C21" t="s">
         <v>135</v>
       </c>
-      <c r="D21" t="e">
-        <f>GETPIVOTDATA("REMAIN",Sheet1!$Q$5,"ACTION PLAN","ACTION PLAN AC#2 WK27","HANDLE","HUAWEI","Years (SO DATE)",2026)</f>
-        <v>#REF!</v>
+      <c r="D21">
+        <f>Sheet1!T13</f>
+        <v>115382.22000000031</v>
       </c>
       <c r="E21" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>133</v>
       </c>
@@ -5534,15 +5543,15 @@
       <c r="C22" t="s">
         <v>140</v>
       </c>
-      <c r="D22" t="e">
+      <c r="D22">
         <f>SUM(D18:D21)</f>
-        <v>#REF!</v>
+        <v>215035.3200000003</v>
       </c>
       <c r="E22" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>142</v>
       </c>
@@ -5566,7 +5575,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>142</v>
       </c>
@@ -5590,7 +5599,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>142</v>
       </c>
@@ -5614,7 +5623,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>142</v>
       </c>
@@ -5638,7 +5647,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>142</v>
       </c>
@@ -5662,7 +5671,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>157</v>
       </c>
@@ -5680,7 +5689,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>157</v>
       </c>
@@ -5698,7 +5707,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>157</v>
       </c>
@@ -5716,7 +5725,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>157</v>
       </c>
@@ -5734,7 +5743,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>157</v>
       </c>
@@ -5752,7 +5761,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>157</v>
       </c>
@@ -5770,7 +5779,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>157</v>
       </c>
@@ -5788,7 +5797,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>157</v>
       </c>
@@ -5806,7 +5815,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>157</v>
       </c>
@@ -5824,7 +5833,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:G36" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:G12 A14:G14 A13:C13 E13:G13 A17:G17 A15:C15 E15:G15 A16:C16 E16:G16 A22:G36 A18:C18 E18:G18 A19:C19 E19:G19 A20:C20 E20:G20 A21:C21 E21:G21" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5832,9 +5841,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5848,7 +5857,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>171</v>
       </c>
@@ -5862,7 +5871,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>175</v>
       </c>
@@ -5887,9 +5896,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5906,7 +5915,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>182</v>
       </c>
@@ -5934,7 +5943,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.5" bestFit="1" customWidth="1"/>
@@ -5946,7 +5955,7 @@
     <col min="11" max="11" width="19.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>187</v>
       </c>
@@ -5975,7 +5984,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -6004,7 +6013,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>190</v>
       </c>
@@ -6039,7 +6048,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>193</v>
       </c>
@@ -6074,7 +6083,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -6109,7 +6118,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -6144,7 +6153,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -6190,9 +6199,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:BP264"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>203</v>
       </c>
@@ -6350,7 +6359,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="2" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A2">
         <f>SUBTOTAL(3,A4:A9935)</f>
         <v>252</v>
@@ -6592,7 +6601,7 @@
         <v>2370096.08</v>
       </c>
     </row>
-    <row r="3" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>206</v>
       </c>
@@ -6795,7 +6804,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="4" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>29753</v>
       </c>
@@ -6990,7 +6999,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="5" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>29754</v>
       </c>
@@ -7185,7 +7194,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="6" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>29762</v>
       </c>
@@ -7380,7 +7389,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="7" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>29763</v>
       </c>
@@ -7572,7 +7581,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="8" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>29767</v>
       </c>
@@ -7767,7 +7776,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="9" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>29725</v>
       </c>
@@ -7962,7 +7971,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="10" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>29757</v>
       </c>
@@ -8157,7 +8166,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="11" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>29758</v>
       </c>
@@ -8352,7 +8361,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="12" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>29759</v>
       </c>
@@ -8547,7 +8556,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="13" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>29760</v>
       </c>
@@ -8742,7 +8751,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="14" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>29761</v>
       </c>
@@ -8934,7 +8943,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="15" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>29764</v>
       </c>
@@ -9129,7 +9138,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="16" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>29766</v>
       </c>
@@ -9321,7 +9330,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="17" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>29755</v>
       </c>
@@ -9516,7 +9525,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="18" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>29765</v>
       </c>
@@ -9708,7 +9717,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="19" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>336</v>
       </c>
@@ -9903,7 +9912,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="20" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>341</v>
       </c>
@@ -10092,7 +10101,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="21" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>349</v>
       </c>
@@ -10281,7 +10290,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="22" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>353</v>
       </c>
@@ -10470,7 +10479,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="23" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>357</v>
       </c>
@@ -10659,7 +10668,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="24" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>361</v>
       </c>
@@ -10848,7 +10857,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="25" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>368</v>
       </c>
@@ -11037,7 +11046,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="26" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>372</v>
       </c>
@@ -11232,7 +11241,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="27" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>376</v>
       </c>
@@ -11427,7 +11436,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="28" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>380</v>
       </c>
@@ -11622,7 +11631,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="29" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>384</v>
       </c>
@@ -11817,7 +11826,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="30" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>388</v>
       </c>
@@ -12009,7 +12018,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="31" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>392</v>
       </c>
@@ -12201,7 +12210,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="32" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>396</v>
       </c>
@@ -12396,7 +12405,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="33" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>401</v>
       </c>
@@ -12591,7 +12600,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="34" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>405</v>
       </c>
@@ -12786,7 +12795,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="35" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>409</v>
       </c>
@@ -12981,7 +12990,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="36" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>413</v>
       </c>
@@ -13173,7 +13182,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="37" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>417</v>
       </c>
@@ -13365,7 +13374,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="38" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>421</v>
       </c>
@@ -13560,7 +13569,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="39" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>425</v>
       </c>
@@ -13749,7 +13758,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="40" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>429</v>
       </c>
@@ -13944,7 +13953,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="41" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>433</v>
       </c>
@@ -14133,7 +14142,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="42" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>437</v>
       </c>
@@ -14322,7 +14331,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="43" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>441</v>
       </c>
@@ -14517,7 +14526,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="44" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>445</v>
       </c>
@@ -14712,7 +14721,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="45" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>449</v>
       </c>
@@ -14907,7 +14916,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="46" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>454</v>
       </c>
@@ -15102,7 +15111,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="47" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>459</v>
       </c>
@@ -15297,7 +15306,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="48" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>463</v>
       </c>
@@ -15492,7 +15501,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="49" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>467</v>
       </c>
@@ -15687,7 +15696,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="50" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>471</v>
       </c>
@@ -15882,7 +15891,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="51" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>475</v>
       </c>
@@ -16077,7 +16086,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="52" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>479</v>
       </c>
@@ -16272,7 +16281,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="53" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>483</v>
       </c>
@@ -16467,7 +16476,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="54" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>487</v>
       </c>
@@ -16653,7 +16662,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="55" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>491</v>
       </c>
@@ -16842,7 +16851,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="56" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>495</v>
       </c>
@@ -17031,7 +17040,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="57" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>499</v>
       </c>
@@ -17220,7 +17229,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="58" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>503</v>
       </c>
@@ -17409,7 +17418,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="59" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>507</v>
       </c>
@@ -17598,7 +17607,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="60" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>511</v>
       </c>
@@ -17787,7 +17796,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="61" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>515</v>
       </c>
@@ -17976,7 +17985,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="62" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>519</v>
       </c>
@@ -18165,7 +18174,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="63" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>523</v>
       </c>
@@ -18354,7 +18363,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="64" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>527</v>
       </c>
@@ -18543,7 +18552,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="65" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>531</v>
       </c>
@@ -18732,7 +18741,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="66" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>535</v>
       </c>
@@ -18921,7 +18930,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="67" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>539</v>
       </c>
@@ -19110,7 +19119,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="68" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>543</v>
       </c>
@@ -19299,7 +19308,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="69" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>547</v>
       </c>
@@ -19488,7 +19497,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="70" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>29509</v>
       </c>
@@ -19614,7 +19623,7 @@
         <v>TREDISMANTLE</v>
       </c>
     </row>
-    <row r="71" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>556</v>
       </c>
@@ -19800,7 +19809,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="72" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>560</v>
       </c>
@@ -19986,7 +19995,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="73" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>564</v>
       </c>
@@ -20172,7 +20181,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="74" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>568</v>
       </c>
@@ -20352,7 +20361,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="75" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>572</v>
       </c>
@@ -20529,7 +20538,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="76" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>576</v>
       </c>
@@ -20706,7 +20715,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="77" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>580</v>
       </c>
@@ -20886,7 +20895,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="78" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>585</v>
       </c>
@@ -21063,7 +21072,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="79" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>590</v>
       </c>
@@ -21243,7 +21252,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="80" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>594</v>
       </c>
@@ -21423,7 +21432,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="81" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>598</v>
       </c>
@@ -21603,7 +21612,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="82" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>602</v>
       </c>
@@ -21783,7 +21792,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="83" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>607</v>
       </c>
@@ -21963,7 +21972,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="84" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>611</v>
       </c>
@@ -22143,7 +22152,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="85" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>615</v>
       </c>
@@ -22323,7 +22332,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="86" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>619</v>
       </c>
@@ -22503,7 +22512,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="87" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>623</v>
       </c>
@@ -22683,7 +22692,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="88" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>627</v>
       </c>
@@ -22863,7 +22872,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="89" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>631</v>
       </c>
@@ -23043,7 +23052,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="90" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>635</v>
       </c>
@@ -23223,7 +23232,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="91" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>639</v>
       </c>
@@ -23403,7 +23412,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="92" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>643</v>
       </c>
@@ -23565,7 +23574,7 @@
         <v>HAECANCEL</v>
       </c>
     </row>
-    <row r="93" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>648</v>
       </c>
@@ -23745,7 +23754,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="94" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>653</v>
       </c>
@@ -23922,7 +23931,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="95" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>658</v>
       </c>
@@ -24099,7 +24108,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="96" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>662</v>
       </c>
@@ -24276,7 +24285,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="97" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>666</v>
       </c>
@@ -24453,7 +24462,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="98" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>670</v>
       </c>
@@ -24630,7 +24639,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="99" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>675</v>
       </c>
@@ -24807,7 +24816,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="100" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>679</v>
       </c>
@@ -24984,7 +24993,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="101" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>683</v>
       </c>
@@ -25161,7 +25170,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="102" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>687</v>
       </c>
@@ -25323,7 +25332,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="103" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>691</v>
       </c>
@@ -25500,7 +25509,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="104" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>695</v>
       </c>
@@ -25653,7 +25662,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="105" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>699</v>
       </c>
@@ -25812,7 +25821,7 @@
         <v>TMECANCEL</v>
       </c>
     </row>
-    <row r="106" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>703</v>
       </c>
@@ -25983,7 +25992,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="107" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>708</v>
       </c>
@@ -26160,7 +26169,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="108" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>712</v>
       </c>
@@ -26337,7 +26346,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="109" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>716</v>
       </c>
@@ -26514,7 +26523,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="110" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>720</v>
       </c>
@@ -26685,7 +26694,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="111" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>723</v>
       </c>
@@ -26862,7 +26871,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="112" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>727</v>
       </c>
@@ -27009,7 +27018,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="113" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>731</v>
       </c>
@@ -27156,7 +27165,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="114" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>735</v>
       </c>
@@ -27333,7 +27342,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="115" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>738</v>
       </c>
@@ -27510,7 +27519,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="116" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:68" x14ac:dyDescent="0.25">
       <c r="B116" t="s">
         <v>742</v>
       </c>
@@ -27621,7 +27630,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="117" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:68" x14ac:dyDescent="0.25">
       <c r="B117" t="s">
         <v>745</v>
       </c>
@@ -27732,7 +27741,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="118" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>748</v>
       </c>
@@ -27879,7 +27888,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="119" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>752</v>
       </c>
@@ -28056,7 +28065,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="120" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>756</v>
       </c>
@@ -28233,7 +28242,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="121" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>760</v>
       </c>
@@ -28407,7 +28416,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="122" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>765</v>
       </c>
@@ -28581,7 +28590,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="123" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>770</v>
       </c>
@@ -28734,7 +28743,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="124" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>774</v>
       </c>
@@ -28875,7 +28884,7 @@
         <v>TMEIPRAN</v>
       </c>
     </row>
-    <row r="125" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>778</v>
       </c>
@@ -29040,7 +29049,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="126" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>783</v>
       </c>
@@ -29205,7 +29214,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="127" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>27555</v>
       </c>
@@ -29340,7 +29349,7 @@
         <v>TMEMBB</v>
       </c>
     </row>
-    <row r="128" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>793</v>
       </c>
@@ -29472,7 +29481,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="129" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>798</v>
       </c>
@@ -29616,7 +29625,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="130" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>803</v>
       </c>
@@ -29763,7 +29772,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="131" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>807</v>
       </c>
@@ -29907,7 +29916,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="132" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>811</v>
       </c>
@@ -30057,7 +30066,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="133" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>815</v>
       </c>
@@ -30204,7 +30213,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="134" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>819</v>
       </c>
@@ -30351,7 +30360,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="135" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>824</v>
       </c>
@@ -30501,7 +30510,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="136" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>828</v>
       </c>
@@ -30651,7 +30660,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="137" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>832</v>
       </c>
@@ -30798,7 +30807,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="138" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>836</v>
       </c>
@@ -30936,7 +30945,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="139" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>841</v>
       </c>
@@ -31041,7 +31050,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="140" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>845</v>
       </c>
@@ -31191,7 +31200,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="141" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>850</v>
       </c>
@@ -31296,7 +31305,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="142" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>854</v>
       </c>
@@ -31401,7 +31410,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="143" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>858</v>
       </c>
@@ -31506,7 +31515,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="144" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>862</v>
       </c>
@@ -31638,7 +31647,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="145" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>866</v>
       </c>
@@ -31788,7 +31797,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="146" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>870</v>
       </c>
@@ -31923,7 +31932,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="147" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>874</v>
       </c>
@@ -32028,7 +32037,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="148" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>878</v>
       </c>
@@ -32133,7 +32142,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="149" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>882</v>
       </c>
@@ -32280,7 +32289,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="150" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>886</v>
       </c>
@@ -32418,7 +32427,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="151" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>890</v>
       </c>
@@ -32559,7 +32568,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="152" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>894</v>
       </c>
@@ -32664,7 +32673,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="153" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>898</v>
       </c>
@@ -32769,7 +32778,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="154" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>902</v>
       </c>
@@ -32874,7 +32883,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="155" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>906</v>
       </c>
@@ -33012,7 +33021,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="156" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>910</v>
       </c>
@@ -33117,7 +33126,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="157" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>914</v>
       </c>
@@ -33222,7 +33231,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="158" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>918</v>
       </c>
@@ -33327,7 +33336,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="159" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>922</v>
       </c>
@@ -33432,7 +33441,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="160" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>926</v>
       </c>
@@ -33537,7 +33546,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="161" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>930</v>
       </c>
@@ -33642,7 +33651,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="162" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>934</v>
       </c>
@@ -33747,7 +33756,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="163" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>938</v>
       </c>
@@ -33852,7 +33861,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="164" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>942</v>
       </c>
@@ -33957,7 +33966,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="165" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>946</v>
       </c>
@@ -34062,7 +34071,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="166" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>950</v>
       </c>
@@ -34197,7 +34206,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="167" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>954</v>
       </c>
@@ -34302,7 +34311,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="168" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>958</v>
       </c>
@@ -34437,7 +34446,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="169" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>962</v>
       </c>
@@ -34542,7 +34551,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="170" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>966</v>
       </c>
@@ -34647,7 +34656,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="171" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>970</v>
       </c>
@@ -34752,7 +34761,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="172" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>974</v>
       </c>
@@ -34884,7 +34893,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="173" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>978</v>
       </c>
@@ -35028,7 +35037,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="174" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>982</v>
       </c>
@@ -35133,7 +35142,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="175" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>986</v>
       </c>
@@ -35274,7 +35283,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="176" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>990</v>
       </c>
@@ -35379,7 +35388,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="177" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>994</v>
       </c>
@@ -35499,7 +35508,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="178" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>998</v>
       </c>
@@ -35604,7 +35613,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="179" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>1002</v>
       </c>
@@ -35754,7 +35763,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="180" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>1006</v>
       </c>
@@ -35859,7 +35868,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="181" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>1010</v>
       </c>
@@ -35964,7 +35973,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="182" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>1014</v>
       </c>
@@ -36096,7 +36105,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="183" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>1018</v>
       </c>
@@ -36201,7 +36210,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="184" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>1022</v>
       </c>
@@ -36306,7 +36315,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="185" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>1026</v>
       </c>
@@ -36411,7 +36420,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="186" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>1030</v>
       </c>
@@ -36516,7 +36525,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="187" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>1034</v>
       </c>
@@ -36621,7 +36630,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="188" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>1038</v>
       </c>
@@ -36726,7 +36735,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="189" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>1042</v>
       </c>
@@ -36831,7 +36840,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="190" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>1046</v>
       </c>
@@ -36936,7 +36945,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="191" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>1050</v>
       </c>
@@ -37041,7 +37050,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="192" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>1054</v>
       </c>
@@ -37170,7 +37179,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="193" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>1058</v>
       </c>
@@ -37302,7 +37311,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="194" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>1062</v>
       </c>
@@ -37431,7 +37440,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="195" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>1066</v>
       </c>
@@ -37536,7 +37545,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="196" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>1068</v>
       </c>
@@ -37665,7 +37674,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="197" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>1072</v>
       </c>
@@ -37770,7 +37779,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="198" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>1076</v>
       </c>
@@ -37875,7 +37884,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="199" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>1079</v>
       </c>
@@ -37995,7 +38004,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="200" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>1083</v>
       </c>
@@ -38127,7 +38136,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="201" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>1087</v>
       </c>
@@ -38232,7 +38241,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="202" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>1091</v>
       </c>
@@ -38337,7 +38346,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="203" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>1095</v>
       </c>
@@ -38442,7 +38451,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="204" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>1099</v>
       </c>
@@ -38562,7 +38571,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="205" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>1103</v>
       </c>
@@ -38691,7 +38700,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="206" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>1107</v>
       </c>
@@ -38796,7 +38805,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="207" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>1111</v>
       </c>
@@ -38916,7 +38925,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="208" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>1114</v>
       </c>
@@ -39021,7 +39030,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="209" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>1118</v>
       </c>
@@ -39126,7 +39135,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="210" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>1121</v>
       </c>
@@ -39246,7 +39255,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="211" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>1125</v>
       </c>
@@ -39351,7 +39360,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="212" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>1129</v>
       </c>
@@ -39483,7 +39492,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="213" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>1132</v>
       </c>
@@ -39603,7 +39612,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="214" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>1135</v>
       </c>
@@ -39708,7 +39717,7 @@
         <v>TMEMBB</v>
       </c>
     </row>
-    <row r="215" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>1140</v>
       </c>
@@ -39813,7 +39822,7 @@
         <v>TMEBATERRY</v>
       </c>
     </row>
-    <row r="216" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>1144</v>
       </c>
@@ -39945,7 +39954,7 @@
         <v>TMEMBB</v>
       </c>
     </row>
-    <row r="217" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>1149</v>
       </c>
@@ -40050,7 +40059,7 @@
         <v>TMEMBB</v>
       </c>
     </row>
-    <row r="218" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:68" x14ac:dyDescent="0.25">
       <c r="B218" t="s">
         <v>1153</v>
       </c>
@@ -40143,7 +40152,7 @@
         <v>TMEMBB</v>
       </c>
     </row>
-    <row r="219" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:68" x14ac:dyDescent="0.25">
       <c r="B219" t="s">
         <v>1156</v>
       </c>
@@ -40236,7 +40245,7 @@
         <v>TMEMBB</v>
       </c>
     </row>
-    <row r="220" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:68" x14ac:dyDescent="0.25">
       <c r="B220" t="s">
         <v>1159</v>
       </c>
@@ -40329,7 +40338,7 @@
         <v>TMEMBB</v>
       </c>
     </row>
-    <row r="221" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>1162</v>
       </c>
@@ -40434,7 +40443,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="222" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>1166</v>
       </c>
@@ -40539,7 +40548,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="223" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>1170</v>
       </c>
@@ -40644,7 +40653,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="224" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>1174</v>
       </c>
@@ -40749,7 +40758,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="225" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>1178</v>
       </c>
@@ -40854,7 +40863,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="226" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>1182</v>
       </c>
@@ -40959,7 +40968,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="227" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>1186</v>
       </c>
@@ -41064,7 +41073,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="228" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>1190</v>
       </c>
@@ -41169,7 +41178,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="229" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>1194</v>
       </c>
@@ -41274,7 +41283,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="230" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>1198</v>
       </c>
@@ -41379,7 +41388,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="231" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>1202</v>
       </c>
@@ -41484,7 +41493,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="232" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>1206</v>
       </c>
@@ -41589,7 +41598,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="233" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>1210</v>
       </c>
@@ -41694,7 +41703,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="234" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>1214</v>
       </c>
@@ -41799,7 +41808,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="235" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>1218</v>
       </c>
@@ -41904,7 +41913,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="236" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>1222</v>
       </c>
@@ -42009,7 +42018,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="237" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>1226</v>
       </c>
@@ -42114,7 +42123,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="238" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>1230</v>
       </c>
@@ -42219,7 +42228,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="239" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>1234</v>
       </c>
@@ -42324,7 +42333,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="240" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>1238</v>
       </c>
@@ -42429,7 +42438,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="241" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>1242</v>
       </c>
@@ -42534,7 +42543,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="242" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>1246</v>
       </c>
@@ -42639,7 +42648,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="243" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>1250</v>
       </c>
@@ -42744,7 +42753,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="244" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>1254</v>
       </c>
@@ -42849,7 +42858,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="245" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>1258</v>
       </c>
@@ -42954,7 +42963,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="246" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>1262</v>
       </c>
@@ -43059,7 +43068,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="247" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>1266</v>
       </c>
@@ -43164,7 +43173,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="248" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>1270</v>
       </c>
@@ -43269,7 +43278,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="249" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>1274</v>
       </c>
@@ -43374,7 +43383,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="250" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>1278</v>
       </c>
@@ -43479,7 +43488,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="251" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>1282</v>
       </c>
@@ -43584,7 +43593,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="252" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>1286</v>
       </c>
@@ -43689,7 +43698,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="253" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>1290</v>
       </c>
@@ -43794,7 +43803,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="254" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>1294</v>
       </c>
@@ -43899,7 +43908,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="255" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>1298</v>
       </c>
@@ -44004,7 +44013,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="256" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>1302</v>
       </c>
@@ -44109,7 +44118,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="257" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>1306</v>
       </c>
@@ -44214,7 +44223,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="258" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>1309</v>
       </c>
@@ -44319,7 +44328,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="259" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>1313</v>
       </c>
@@ -44424,7 +44433,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="260" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>1317</v>
       </c>
@@ -44529,7 +44538,7 @@
         <v>HAEMBB</v>
       </c>
     </row>
-    <row r="261" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:68" x14ac:dyDescent="0.25">
       <c r="B261" t="s">
         <v>1321</v>
       </c>
@@ -44622,7 +44631,7 @@
         <v>TMEMBB</v>
       </c>
     </row>
-    <row r="262" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:68" x14ac:dyDescent="0.25">
       <c r="B262" t="s">
         <v>1324</v>
       </c>
@@ -44715,7 +44724,7 @@
         <v>TMEMBB</v>
       </c>
     </row>
-    <row r="263" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:68" x14ac:dyDescent="0.25">
       <c r="B263" t="s">
         <v>1327</v>
       </c>
@@ -44808,7 +44817,7 @@
         <v>TMEMBB</v>
       </c>
     </row>
-    <row r="264" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:68" x14ac:dyDescent="0.25">
       <c r="B264" t="s">
         <v>1330</v>
       </c>
@@ -44914,9 +44923,28 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="B2:T28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="10.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.75" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.75" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.75" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.75" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="22.625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="19.625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>1333</v>
       </c>
@@ -44930,7 +44958,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="3" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:20" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
         <v>1335</v>
       </c>
@@ -44956,7 +44984,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="4" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>1342</v>
       </c>
@@ -44988,7 +45016,7 @@
         <v>1345</v>
       </c>
     </row>
-    <row r="5" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>1346</v>
       </c>
@@ -45017,7 +45045,7 @@
         <v>1334</v>
       </c>
     </row>
-    <row r="6" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>1347</v>
       </c>
@@ -45070,7 +45098,7 @@
         <v>1349</v>
       </c>
     </row>
-    <row r="7" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>1350</v>
       </c>
@@ -45120,7 +45148,7 @@
         <v>1864614</v>
       </c>
     </row>
-    <row r="8" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>1352</v>
       </c>
@@ -45170,7 +45198,7 @@
         <v>1864614</v>
       </c>
     </row>
-    <row r="9" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>1353</v>
       </c>
@@ -45220,7 +45248,7 @@
         <v>215035.3200000003</v>
       </c>
     </row>
-    <row r="10" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>1349</v>
       </c>
@@ -45270,7 +45298,7 @@
         <v>43613.1</v>
       </c>
     </row>
-    <row r="11" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:20" x14ac:dyDescent="0.25">
       <c r="Q11" t="s">
         <v>1350</v>
       </c>
@@ -45281,7 +45309,7 @@
         <v>12891.900000000001</v>
       </c>
     </row>
-    <row r="12" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>1355</v>
       </c>
@@ -45298,7 +45326,7 @@
         <v>43148.100000000013</v>
       </c>
     </row>
-    <row r="13" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:20" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
         <v>1335</v>
       </c>
@@ -45327,7 +45355,7 @@
         <v>115382.22000000031</v>
       </c>
     </row>
-    <row r="14" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>1342</v>
       </c>
@@ -45371,7 +45399,7 @@
         <v>430719.4</v>
       </c>
     </row>
-    <row r="15" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>1346</v>
       </c>
@@ -45403,7 +45431,7 @@
         <v>80317</v>
       </c>
     </row>
-    <row r="16" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>1347</v>
       </c>
@@ -45453,7 +45481,7 @@
         <v>60400</v>
       </c>
     </row>
-    <row r="17" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>1350</v>
       </c>
@@ -45494,7 +45522,7 @@
         <v>53562</v>
       </c>
     </row>
-    <row r="18" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>1352</v>
       </c>
@@ -45547,7 +45575,7 @@
         <v>236440.4</v>
       </c>
     </row>
-    <row r="19" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>1353</v>
       </c>
@@ -45597,7 +45625,7 @@
         <v>64754.400000000001</v>
       </c>
     </row>
-    <row r="20" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>1349</v>
       </c>
@@ -45647,7 +45675,7 @@
         <v>10369.500000000002</v>
       </c>
     </row>
-    <row r="21" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:20" x14ac:dyDescent="0.25">
       <c r="Q21" t="s">
         <v>1352</v>
       </c>
@@ -45658,7 +45686,7 @@
         <v>13164.900000000001</v>
       </c>
     </row>
-    <row r="22" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:20" x14ac:dyDescent="0.25">
       <c r="Q22" t="s">
         <v>1353</v>
       </c>
@@ -45669,7 +45697,7 @@
         <v>41220</v>
       </c>
     </row>
-    <row r="23" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:20" x14ac:dyDescent="0.25">
       <c r="Q23" t="s">
         <v>1349</v>
       </c>
@@ -45683,7 +45711,7 @@
         <v>2575123.12</v>
       </c>
     </row>
-    <row r="25" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:20" x14ac:dyDescent="0.25">
       <c r="Q25">
         <v>2023</v>
       </c>
@@ -45692,7 +45720,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="26" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
       <c r="Q26">
         <v>2024</v>
       </c>
@@ -45701,7 +45729,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="27" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:20" x14ac:dyDescent="0.25">
       <c r="Q27">
         <v>2025</v>
       </c>
@@ -45710,7 +45738,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="28" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:20" x14ac:dyDescent="0.25">
       <c r="Q28">
         <v>2026</v>
       </c>

</xml_diff>

<commit_message>
Fix Excel data import parsing for Backlog, Milestone Aging, SO Comparison, and SLA
</commit_message>
<xml_diff>
--- a/Dashboard_Template_30_Slides_Final.xlsx
+++ b/Dashboard_Template_30_Slides_Final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\0_Dashboad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BB65F4E-4CD7-465D-B29A-F5DB56BB046B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{892BEE5C-8B2A-42B0-906A-7973899F9AFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="791" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="791" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Part 1 - Overview" sheetId="1" r:id="rId1"/>
@@ -199,7 +199,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5099" uniqueCount="1388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5122" uniqueCount="1389">
   <si>
     <t>Slide No</t>
   </si>
@@ -4356,13 +4356,16 @@
     <t>2 วัน</t>
   </si>
   <si>
-    <t>No rework required 🎉</t>
-  </si>
-  <si>
     <t>Backlog Week 28</t>
   </si>
   <si>
     <t>Backlog Backlog Week 27 VS Backlog Week 28</t>
+  </si>
+  <si>
+    <t>1 วัน</t>
+  </si>
+  <si>
+    <t>6 วัน</t>
   </si>
 </sst>
 </file>
@@ -4521,13 +4524,14 @@
       <family val="2"/>
     </font>
     <font>
+      <b/>
       <sz val="10"/>
-      <color rgb="FF15803D"/>
+      <color rgb="FFEA580C"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4624,8 +4628,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEDD5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="19">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -4825,6 +4835,19 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCBD5E1"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCBD5E1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFCBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -4833,7 +4856,7 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5053,17 +5076,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="15" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="16" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="43" fontId="0" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="19" fillId="11" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -5085,8 +5104,33 @@
     <xf numFmtId="0" fontId="17" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="43" fontId="0" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -5486,7 +5530,7 @@
       </c>
       <c r="D3" s="59">
         <f>'Part 2 - Aging'!D3</f>
-        <v>1.5476190476190477</v>
+        <v>1.5568862275449102</v>
       </c>
       <c r="E3" t="s">
         <v>11</v>
@@ -5644,7 +5688,7 @@
       </c>
       <c r="D3" s="59">
         <f>AVERAGEIF('2026'!G:G,"HAE",'2026'!BD:BD)</f>
-        <v>1.5476190476190477</v>
+        <v>1.5568862275449102</v>
       </c>
       <c r="E3" t="s">
         <v>1333</v>
@@ -5662,7 +5706,7 @@
       </c>
       <c r="D4" s="59">
         <f>AVERAGEIF('2026'!G:G,"HAE",'2026'!BE:BE)</f>
-        <v>3.6706586826347305</v>
+        <v>3.6927710843373496</v>
       </c>
       <c r="E4" t="s">
         <v>1335</v>
@@ -5731,7 +5775,7 @@
       </c>
       <c r="D8" s="59">
         <f>AVERAGE(D3:D4)</f>
-        <v>2.609138865126889</v>
+        <v>2.6248286559411298</v>
       </c>
       <c r="E8" t="s">
         <v>46</v>
@@ -5749,7 +5793,7 @@
       </c>
       <c r="D9" s="59">
         <f>AVERAGE(D4:D5)</f>
-        <v>2.6653293413173653</v>
+        <v>2.6763855421686746</v>
       </c>
       <c r="E9" t="s">
         <v>46</v>
@@ -5767,7 +5811,7 @@
       </c>
       <c r="D10" s="59">
         <f>AVERAGEIF('2026'!R:R,"Palagon Prommueangma",'2026'!BD:BD)</f>
-        <v>1.7857142857142858</v>
+        <v>1.9230769230769231</v>
       </c>
       <c r="E10" t="s">
         <v>46</v>
@@ -5968,7 +6012,7 @@
       </c>
       <c r="D7">
         <f>'2026'!AB2*0.7</f>
-        <v>2681227.7799999998</v>
+        <v>2684751.5799999996</v>
       </c>
       <c r="E7">
         <f>'2026'!BH2</f>
@@ -5976,7 +6020,7 @@
       </c>
       <c r="F7" s="59">
         <f>AVERAGE('2026'!BJ4:BJ260)</f>
-        <v>10.62809917355372</v>
+        <v>10.716666666666667</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -5991,7 +6035,7 @@
       </c>
       <c r="D8">
         <f>'2026'!AB2*0.3</f>
-        <v>1149097.6199999999</v>
+        <v>1150607.8199999998</v>
       </c>
       <c r="E8">
         <f>'2026'!BK2</f>
@@ -5999,7 +6043,7 @@
       </c>
       <c r="F8" s="59">
         <f>AVERAGE('2026'!BM4:BM260)</f>
-        <v>14.74375</v>
+        <v>14.930379746835444</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -6073,7 +6117,7 @@
       </c>
       <c r="D2" s="58">
         <f>'2026'!AB2</f>
-        <v>3830325.4</v>
+        <v>3835359.4</v>
       </c>
       <c r="E2" t="s">
         <v>85</v>
@@ -6127,7 +6171,7 @@
       </c>
       <c r="D5" s="58">
         <f>D2-(D3+D4)</f>
-        <v>2482944.9800000014</v>
+        <v>2487978.9800000014</v>
       </c>
       <c r="E5" t="s">
         <v>95</v>
@@ -6138,7 +6182,7 @@
         <v>55</v>
       </c>
       <c r="B6" t="s">
-        <v>1387</v>
+        <v>1386</v>
       </c>
       <c r="C6" t="s">
         <v>97</v>
@@ -6156,10 +6200,10 @@
         <v>55</v>
       </c>
       <c r="B7" t="s">
-        <v>1387</v>
+        <v>1386</v>
       </c>
       <c r="C7" t="s">
-        <v>1386</v>
+        <v>1385</v>
       </c>
       <c r="D7" s="58">
         <f>Sheet1!N20</f>
@@ -6221,19 +6265,19 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="87" t="s">
+      <c r="A11" s="78" t="s">
         <v>58</v>
       </c>
-      <c r="B11" s="87" t="s">
+      <c r="B11" s="78" t="s">
         <v>1325</v>
       </c>
-      <c r="C11" s="87" t="s">
+      <c r="C11" s="78" t="s">
         <v>1325</v>
       </c>
-      <c r="D11" s="88">
+      <c r="D11" s="79">
         <v>197419.3</v>
       </c>
-      <c r="E11" s="87" t="s">
+      <c r="E11" s="78" t="s">
         <v>1347</v>
       </c>
     </row>
@@ -6272,54 +6316,54 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="87" t="s">
+      <c r="A14" s="78" t="s">
         <v>66</v>
       </c>
-      <c r="B14" s="87" t="s">
+      <c r="B14" s="78" t="s">
         <v>1356</v>
       </c>
-      <c r="C14" s="87" t="s">
+      <c r="C14" s="78" t="s">
         <v>105</v>
       </c>
-      <c r="D14" s="88">
+      <c r="D14" s="79">
         <v>64754</v>
       </c>
-      <c r="E14" s="87" t="s">
+      <c r="E14" s="78" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="87" t="s">
+      <c r="A15" s="78" t="s">
         <v>66</v>
       </c>
-      <c r="B15" s="87" t="s">
+      <c r="B15" s="78" t="s">
         <v>1357</v>
       </c>
-      <c r="C15" s="87" t="s">
+      <c r="C15" s="78" t="s">
         <v>111</v>
       </c>
-      <c r="D15" s="88">
+      <c r="D15" s="79">
         <v>215035</v>
       </c>
-      <c r="E15" s="87" t="s">
+      <c r="E15" s="78" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="87" t="s">
+      <c r="A16" s="78" t="s">
         <v>66</v>
       </c>
-      <c r="B16" s="87" t="s">
+      <c r="B16" s="78" t="s">
         <v>1368</v>
       </c>
-      <c r="C16" s="87" t="s">
+      <c r="C16" s="78" t="s">
         <v>1369</v>
       </c>
-      <c r="D16" s="88">
+      <c r="D16" s="79">
         <f>SUM(D14:D15)</f>
         <v>279789</v>
       </c>
-      <c r="E16" s="87" t="s">
+      <c r="E16" s="78" t="s">
         <v>1369</v>
       </c>
     </row>
@@ -6586,7 +6630,7 @@
       </c>
       <c r="D30" s="58">
         <f>SUMIF('2026'!BP:BP,'Part 4 - Financials'!F30&amp;'Part 4 - Financials'!G30,'2026'!AB:AB)</f>
-        <v>3338143</v>
+        <v>3343177</v>
       </c>
       <c r="E30" t="s">
         <v>116</v>
@@ -6893,7 +6937,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.125" bestFit="1" customWidth="1"/>
@@ -6907,7 +6951,7 @@
     <col min="13" max="13" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="17.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="82" t="s">
         <v>1370</v>
       </c>
@@ -6946,7 +6990,7 @@
         <v>1375</v>
       </c>
       <c r="B3" s="62">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C3" s="63">
         <v>0.7</v>
@@ -6956,7 +7000,7 @@
         <v>1376</v>
       </c>
       <c r="F3" s="62">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G3" s="63">
         <v>3</v>
@@ -6988,20 +7032,20 @@
         <v>1379</v>
       </c>
       <c r="B5" s="62">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C5" s="63">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="D5" s="60"/>
       <c r="E5" s="64" t="s">
         <v>1380</v>
       </c>
       <c r="F5" s="62">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" s="63">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -7059,7 +7103,7 @@
       </c>
       <c r="C23" s="69"/>
       <c r="D23" s="74"/>
-      <c r="E23" s="73" t="s">
+      <c r="E23" s="72" t="s">
         <v>158</v>
       </c>
       <c r="F23" s="73" t="s">
@@ -7069,7 +7113,7 @@
         <v>160</v>
       </c>
       <c r="H23" s="74"/>
-      <c r="I23" s="73" t="s">
+      <c r="I23" s="72" t="s">
         <v>158</v>
       </c>
       <c r="J23" s="73" t="s">
@@ -7079,40 +7123,103 @@
         <v>160</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="80" t="s">
-        <v>1383</v>
-      </c>
-      <c r="B24" s="81"/>
+    <row r="24" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="87" t="s">
+        <v>909</v>
+      </c>
+      <c r="B24" s="88" t="s">
+        <v>1384</v>
+      </c>
       <c r="C24" s="69"/>
       <c r="D24" s="74"/>
-      <c r="E24" s="76" t="s">
+      <c r="E24" s="80" t="s">
+        <v>1383</v>
+      </c>
+      <c r="F24" s="81"/>
+      <c r="G24" s="77"/>
+      <c r="H24" s="74"/>
+      <c r="I24" s="90" t="s">
+        <v>949</v>
+      </c>
+      <c r="J24" s="91" t="s">
+        <v>1387</v>
+      </c>
+      <c r="K24" s="94" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="87" t="s">
+        <v>929</v>
+      </c>
+      <c r="B25" s="88" t="s">
+        <v>1384</v>
+      </c>
+      <c r="I25" s="90" t="s">
         <v>973</v>
       </c>
-      <c r="F24" s="77" t="s">
+      <c r="J25" s="91" t="s">
         <v>1384</v>
       </c>
-      <c r="G24" s="78" t="s">
+      <c r="K25" s="94" t="s">
         <v>163</v>
       </c>
-      <c r="H24" s="74"/>
-      <c r="I24" s="80" t="s">
-        <v>1385</v>
-      </c>
-      <c r="J24" s="81"/>
-      <c r="K24" s="79" t="s">
-        <v>245</v>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="87" t="s">
+        <v>957</v>
+      </c>
+      <c r="B26" s="88" t="s">
+        <v>1387</v>
+      </c>
+      <c r="I26" s="90" t="s">
+        <v>881</v>
+      </c>
+      <c r="J26" s="91" t="s">
+        <v>1388</v>
+      </c>
+      <c r="K26" s="94" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="89" t="s">
+        <v>865</v>
+      </c>
+      <c r="B27" s="76" t="s">
+        <v>1387</v>
+      </c>
+      <c r="I27" s="90" t="s">
+        <v>161</v>
+      </c>
+      <c r="J27" s="91" t="s">
+        <v>1388</v>
+      </c>
+      <c r="K27" s="94" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="69"/>
+      <c r="B28" s="69"/>
+      <c r="I28" s="92" t="s">
+        <v>817</v>
+      </c>
+      <c r="J28" s="93" t="s">
+        <v>1384</v>
+      </c>
+      <c r="K28" s="95" t="s">
+        <v>163</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="I24:J24"/>
+  <mergeCells count="6">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="E1:G1"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="E22:F22"/>
     <mergeCell ref="I22:J22"/>
+    <mergeCell ref="E24:F24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7453,7 +7560,7 @@
       </c>
       <c r="AB2" s="13">
         <f t="shared" ref="AB2:AI2" si="0">SUBTOTAL(9,AB4:AB264)</f>
-        <v>3830325.4</v>
+        <v>3835359.4</v>
       </c>
       <c r="AC2" s="13">
         <f t="shared" si="0"/>
@@ -7551,7 +7658,10 @@
       <c r="BC2" s="10"/>
       <c r="BD2" s="10"/>
       <c r="BE2" s="10"/>
-      <c r="BF2" s="10"/>
+      <c r="BF2" s="10">
+        <f>SUBTOTAL(3,BF4:BF264)</f>
+        <v>261</v>
+      </c>
       <c r="BG2" s="10"/>
       <c r="BH2" s="10">
         <f>SUBTOTAL(9,BH4:BH264)</f>
@@ -34537,13 +34647,13 @@
         <v>18672</v>
       </c>
       <c r="Z139" s="39">
-        <v>4319</v>
+        <v>4232</v>
       </c>
       <c r="AA139" s="43">
         <v>46207</v>
       </c>
       <c r="AB139" s="39">
-        <v>22991</v>
+        <v>22904</v>
       </c>
       <c r="AC139" s="39">
         <v>11576.64</v>
@@ -34644,7 +34754,7 @@
         <v>0</v>
       </c>
       <c r="BO139" s="49">
-        <v>22991</v>
+        <v>22904</v>
       </c>
       <c r="BP139" t="str">
         <f t="shared" si="4"/>
@@ -34884,10 +34994,14 @@
       <c r="K141" s="37" t="s">
         <v>243</v>
       </c>
-      <c r="L141" s="41"/>
-      <c r="M141" s="41"/>
+      <c r="L141" s="41">
+        <v>46206</v>
+      </c>
+      <c r="M141" s="41">
+        <v>46208</v>
+      </c>
       <c r="N141" s="42">
-        <v>0</v>
+        <v>46208</v>
       </c>
       <c r="O141" s="37" t="s">
         <v>262</v>
@@ -34901,9 +35015,11 @@
       <c r="R141" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="S141" s="37"/>
-      <c r="T141" s="37">
-        <v>0</v>
+      <c r="S141" s="37" t="s">
+        <v>163</v>
+      </c>
+      <c r="T141" s="37" t="s">
+        <v>1322</v>
       </c>
       <c r="U141" s="35">
         <v>779</v>
@@ -34921,11 +35037,11 @@
         <v>20554</v>
       </c>
       <c r="Z141" s="39">
-        <v>0</v>
+        <v>5395</v>
       </c>
       <c r="AA141" s="43"/>
       <c r="AB141" s="39">
-        <v>20554</v>
+        <v>25949</v>
       </c>
       <c r="AC141" s="39">
         <v>12743.48</v>
@@ -34966,12 +35082,8 @@
       <c r="BA141" s="48"/>
       <c r="BB141" s="37"/>
       <c r="BC141" s="37"/>
-      <c r="BD141" s="37">
-        <v>0</v>
-      </c>
-      <c r="BE141" s="37">
-        <v>0</v>
-      </c>
+      <c r="BD141" s="37"/>
+      <c r="BE141" s="37"/>
       <c r="BF141" s="36" t="s">
         <v>250</v>
       </c>
@@ -34982,21 +35094,17 @@
         <v>0</v>
       </c>
       <c r="BI141" s="45"/>
-      <c r="BJ141" s="37">
-        <v>0</v>
-      </c>
+      <c r="BJ141" s="37"/>
       <c r="BK141" s="38">
         <v>0</v>
       </c>
       <c r="BL141" s="45"/>
-      <c r="BM141" s="37">
-        <v>0</v>
-      </c>
+      <c r="BM141" s="37"/>
       <c r="BN141" s="49">
         <v>0</v>
       </c>
       <c r="BO141" s="49">
-        <v>20554</v>
+        <v>25949</v>
       </c>
       <c r="BP141" t="str">
         <f t="shared" si="4"/>
@@ -38606,7 +38714,9 @@
       <c r="R164" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="S164" s="37"/>
+      <c r="S164" s="37" t="s">
+        <v>163</v>
+      </c>
       <c r="T164" s="37" t="s">
         <v>1322</v>
       </c>
@@ -41268,7 +41378,9 @@
       <c r="R180" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="S180" s="37"/>
+      <c r="S180" s="37" t="s">
+        <v>163</v>
+      </c>
       <c r="T180" s="37" t="s">
         <v>1322</v>
       </c>
@@ -44295,13 +44407,13 @@
         <v>33005</v>
       </c>
       <c r="Z199" s="39">
-        <v>16220</v>
+        <v>15946</v>
       </c>
       <c r="AA199" s="43">
         <v>46202</v>
       </c>
       <c r="AB199" s="39">
-        <v>49225</v>
+        <v>48951</v>
       </c>
       <c r="AC199" s="39">
         <v>20463.099999999999</v>
@@ -44402,7 +44514,7 @@
         <v>0</v>
       </c>
       <c r="BO199" s="49">
-        <v>49225</v>
+        <v>48951</v>
       </c>
       <c r="BP199" t="str">
         <f t="shared" si="5"/>
@@ -46803,7 +46915,9 @@
       <c r="K214" s="37" t="s">
         <v>243</v>
       </c>
-      <c r="L214" s="41"/>
+      <c r="L214" s="41">
+        <v>46210</v>
+      </c>
       <c r="M214" s="41"/>
       <c r="N214" s="42">
         <v>0</v>
@@ -47283,9 +47397,11 @@
       <c r="L217" s="41">
         <v>46204</v>
       </c>
-      <c r="M217" s="41"/>
+      <c r="M217" s="41">
+        <v>46208</v>
+      </c>
       <c r="N217" s="42">
-        <v>0</v>
+        <v>46208</v>
       </c>
       <c r="O217" s="37" t="s">
         <v>423</v>
@@ -47302,8 +47418,8 @@
       <c r="S217" s="37" t="s">
         <v>1113</v>
       </c>
-      <c r="T217" s="37">
-        <v>0</v>
+      <c r="T217" s="37" t="s">
+        <v>1322</v>
       </c>
       <c r="U217" s="35">
         <v>0</v>
@@ -47364,14 +47480,10 @@
       <c r="BA217" s="48"/>
       <c r="BB217" s="37"/>
       <c r="BC217" s="37"/>
-      <c r="BD217" s="37">
-        <v>0</v>
-      </c>
-      <c r="BE217" s="37">
-        <v>0</v>
-      </c>
+      <c r="BD217" s="37"/>
+      <c r="BE217" s="37"/>
       <c r="BF217" s="37" t="s">
-        <v>809</v>
+        <v>250</v>
       </c>
       <c r="BG217" s="37" t="s">
         <v>118</v>
@@ -47380,16 +47492,12 @@
         <v>0</v>
       </c>
       <c r="BI217" s="45"/>
-      <c r="BJ217" s="37">
-        <v>0</v>
-      </c>
+      <c r="BJ217" s="37"/>
       <c r="BK217" s="38">
         <v>0</v>
       </c>
       <c r="BL217" s="45"/>
-      <c r="BM217" s="37">
-        <v>0</v>
-      </c>
+      <c r="BM217" s="37"/>
       <c r="BN217" s="49">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Update Dashboard Excel template
</commit_message>
<xml_diff>
--- a/Dashboard_Template_30_Slides_Final.xlsx
+++ b/Dashboard_Template_30_Slides_Final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\0_Dashboad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{892BEE5C-8B2A-42B0-906A-7973899F9AFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D99C1AFC-0B06-43E1-BFFB-D2A7B0C0C610}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="791" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="791" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Part 1 - Overview" sheetId="1" r:id="rId1"/>
@@ -4531,7 +4531,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4631,6 +4631,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEDD5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -4856,7 +4862,7 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5083,27 +5089,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="43" fontId="0" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="15" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -5131,6 +5116,28 @@
     <xf numFmtId="0" fontId="21" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -6952,17 +6959,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="17.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="82" t="s">
+      <c r="A1" s="89" t="s">
         <v>1370</v>
       </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="84"/>
+      <c r="B1" s="90"/>
+      <c r="C1" s="91"/>
       <c r="D1" s="60"/>
-      <c r="E1" s="82" t="s">
+      <c r="E1" s="89" t="s">
         <v>1371</v>
       </c>
-      <c r="F1" s="83"/>
-      <c r="G1" s="84"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="91"/>
     </row>
     <row r="2" spans="1:7" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="61" t="s">
@@ -7072,24 +7079,24 @@
     <row r="7" spans="1:7" ht="16.5" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="22" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="85" t="s">
+      <c r="A22" s="92" t="s">
         <v>155</v>
       </c>
-      <c r="B22" s="86"/>
+      <c r="B22" s="93"/>
       <c r="C22" s="69"/>
       <c r="D22" s="70"/>
-      <c r="E22" s="85" t="s">
+      <c r="E22" s="92" t="s">
         <v>156</v>
       </c>
-      <c r="F22" s="86"/>
+      <c r="F22" s="93"/>
       <c r="G22" s="71" t="s">
         <v>1382</v>
       </c>
       <c r="H22" s="70"/>
-      <c r="I22" s="85" t="s">
+      <c r="I22" s="92" t="s">
         <v>157</v>
       </c>
-      <c r="J22" s="86"/>
+      <c r="J22" s="93"/>
       <c r="K22" s="71" t="s">
         <v>1382</v>
       </c>
@@ -7124,102 +7131,102 @@
       </c>
     </row>
     <row r="24" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="87" t="s">
+      <c r="A24" s="80" t="s">
         <v>909</v>
       </c>
-      <c r="B24" s="88" t="s">
+      <c r="B24" s="81" t="s">
         <v>1384</v>
       </c>
       <c r="C24" s="69"/>
       <c r="D24" s="74"/>
-      <c r="E24" s="80" t="s">
+      <c r="E24" s="94" t="s">
         <v>1383</v>
       </c>
-      <c r="F24" s="81"/>
+      <c r="F24" s="95"/>
       <c r="G24" s="77"/>
       <c r="H24" s="74"/>
-      <c r="I24" s="90" t="s">
+      <c r="I24" s="83" t="s">
         <v>949</v>
       </c>
-      <c r="J24" s="91" t="s">
+      <c r="J24" s="84" t="s">
         <v>1387</v>
       </c>
-      <c r="K24" s="94" t="s">
+      <c r="K24" s="87" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="87" t="s">
+      <c r="A25" s="80" t="s">
         <v>929</v>
       </c>
-      <c r="B25" s="88" t="s">
+      <c r="B25" s="81" t="s">
         <v>1384</v>
       </c>
-      <c r="I25" s="90" t="s">
+      <c r="I25" s="83" t="s">
         <v>973</v>
       </c>
-      <c r="J25" s="91" t="s">
+      <c r="J25" s="84" t="s">
         <v>1384</v>
       </c>
-      <c r="K25" s="94" t="s">
+      <c r="K25" s="87" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" s="87" t="s">
+      <c r="A26" s="80" t="s">
         <v>957</v>
       </c>
-      <c r="B26" s="88" t="s">
+      <c r="B26" s="81" t="s">
         <v>1387</v>
       </c>
-      <c r="I26" s="90" t="s">
+      <c r="I26" s="83" t="s">
         <v>881</v>
       </c>
-      <c r="J26" s="91" t="s">
+      <c r="J26" s="84" t="s">
         <v>1388</v>
       </c>
-      <c r="K26" s="94" t="s">
+      <c r="K26" s="87" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="89" t="s">
+      <c r="A27" s="82" t="s">
         <v>865</v>
       </c>
       <c r="B27" s="76" t="s">
         <v>1387</v>
       </c>
-      <c r="I27" s="90" t="s">
+      <c r="I27" s="83" t="s">
         <v>161</v>
       </c>
-      <c r="J27" s="91" t="s">
+      <c r="J27" s="84" t="s">
         <v>1388</v>
       </c>
-      <c r="K27" s="94" t="s">
+      <c r="K27" s="87" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="69"/>
       <c r="B28" s="69"/>
-      <c r="I28" s="92" t="s">
+      <c r="I28" s="85" t="s">
         <v>817</v>
       </c>
-      <c r="J28" s="93" t="s">
+      <c r="J28" s="86" t="s">
         <v>1384</v>
       </c>
-      <c r="K28" s="95" t="s">
+      <c r="K28" s="88" t="s">
         <v>163</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="E24:F24"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="E1:G1"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="E22:F22"/>
     <mergeCell ref="I22:J22"/>
-    <mergeCell ref="E24:F24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -54243,7 +54250,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
+      <c r="B2" s="96" t="s">
         <v>1319</v>
       </c>
       <c r="C2" t="s">
@@ -54257,13 +54264,13 @@
       </c>
     </row>
     <row r="3" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="C3" t="s">
+      <c r="C3" s="96" t="s">
         <v>1299</v>
       </c>
       <c r="F3" t="s">
         <v>1300</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="96" t="s">
         <v>1301</v>
       </c>
       <c r="L3" t="s">
@@ -54272,7 +54279,7 @@
       <c r="M3" t="s">
         <v>1303</v>
       </c>
-      <c r="N3" t="s">
+      <c r="N3" s="96" t="s">
         <v>1304</v>
       </c>
       <c r="Q3" t="s">
@@ -54292,7 +54299,7 @@
       <c r="D4" t="s">
         <v>1308</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="96" t="s">
         <v>1309</v>
       </c>
       <c r="F4" t="s">
@@ -54310,7 +54317,7 @@
       <c r="J4" t="s">
         <v>1308</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4" s="96" t="s">
         <v>1309</v>
       </c>
     </row>
@@ -54547,7 +54554,7 @@
       <c r="D10">
         <v>332286</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="96">
         <v>109935.79999999997</v>
       </c>
       <c r="F10">
@@ -54565,7 +54572,7 @@
       <c r="J10">
         <v>2250152</v>
       </c>
-      <c r="K10">
+      <c r="K10" s="96">
         <v>2250152</v>
       </c>
       <c r="L10">
@@ -54574,7 +54581,7 @@
       <c r="M10">
         <v>46100400.870000027</v>
       </c>
-      <c r="N10">
+      <c r="N10" s="96">
         <v>2360087.7999999998</v>
       </c>
       <c r="Q10" t="s">
@@ -54599,7 +54606,7 @@
       </c>
     </row>
     <row r="12" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
+      <c r="B12" s="96" t="s">
         <v>1352</v>
       </c>
       <c r="C12" t="s">
@@ -54616,13 +54623,13 @@
       </c>
     </row>
     <row r="13" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="C13" t="s">
+      <c r="C13" s="96" t="s">
         <v>1299</v>
       </c>
       <c r="F13" t="s">
         <v>1300</v>
       </c>
-      <c r="I13" t="s">
+      <c r="I13" s="96" t="s">
         <v>1301</v>
       </c>
       <c r="L13" t="s">
@@ -54631,7 +54638,7 @@
       <c r="M13" t="s">
         <v>1303</v>
       </c>
-      <c r="N13" t="s">
+      <c r="N13" s="96" t="s">
         <v>1304</v>
       </c>
       <c r="Q13" t="s">
@@ -54654,7 +54661,7 @@
       <c r="D14" t="s">
         <v>1308</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="96" t="s">
         <v>1309</v>
       </c>
       <c r="F14" t="s">
@@ -54672,7 +54679,7 @@
       <c r="J14" t="s">
         <v>1308</v>
       </c>
-      <c r="K14" t="s">
+      <c r="K14" s="96" t="s">
         <v>1309</v>
       </c>
       <c r="Q14" t="s">
@@ -54933,7 +54940,7 @@
       <c r="D20">
         <v>513834</v>
       </c>
-      <c r="E20">
+      <c r="E20" s="96">
         <v>147353.47999999995</v>
       </c>
       <c r="F20">
@@ -54951,7 +54958,7 @@
       <c r="J20">
         <v>2163172</v>
       </c>
-      <c r="K20">
+      <c r="K20" s="96">
         <v>2163172</v>
       </c>
       <c r="L20">
@@ -54960,7 +54967,7 @@
       <c r="M20">
         <v>46126843.870000027</v>
       </c>
-      <c r="N20">
+      <c r="N20" s="96">
         <v>2468597.1</v>
       </c>
       <c r="Q20" t="s">

</xml_diff>

<commit_message>
fix: repair brace balance and wire up Financial/AC data to UI
</commit_message>
<xml_diff>
--- a/Dashboard_Template_30_Slides_Final.xlsx
+++ b/Dashboard_Template_30_Slides_Final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\0_Dashboad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C81D2A1E-D523-4E4C-8D5C-3375E064E05F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5600E89F-81C5-45C5-9129-52F1459FF37F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="813" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="813" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Part 1 - Overview" sheetId="1" r:id="rId1"/>
@@ -6017,7 +6017,7 @@
       </c>
       <c r="F8" s="50">
         <f>AVERAGE('2026'!BM4:BM259)</f>
-        <v>-567.87898089171972</v>
+        <v>21.103225806451611</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -7465,63 +7465,63 @@
         <v>3695043.4</v>
       </c>
       <c r="F2" s="10">
-        <f>SUBTOTAL(3,F4:F263)</f>
+        <f t="shared" ref="F2:T2" si="0">SUBTOTAL(3,F4:F263)</f>
         <v>256</v>
       </c>
       <c r="G2" s="10">
-        <f>SUBTOTAL(3,G4:G263)</f>
+        <f t="shared" si="0"/>
         <v>260</v>
       </c>
       <c r="H2" s="10">
-        <f>SUBTOTAL(3,H4:H263)</f>
+        <f t="shared" si="0"/>
         <v>260</v>
       </c>
       <c r="I2" s="10">
-        <f>SUBTOTAL(3,I4:I263)</f>
+        <f t="shared" si="0"/>
         <v>260</v>
       </c>
       <c r="J2" s="10">
-        <f>SUBTOTAL(3,J4:J263)</f>
+        <f t="shared" si="0"/>
         <v>260</v>
       </c>
       <c r="K2" s="10">
-        <f>SUBTOTAL(3,K4:K263)</f>
+        <f t="shared" si="0"/>
         <v>260</v>
       </c>
       <c r="L2" s="10">
-        <f>SUBTOTAL(3,L4:L263)</f>
+        <f t="shared" si="0"/>
         <v>187</v>
       </c>
       <c r="M2" s="10">
-        <f>SUBTOTAL(3,M4:M263)</f>
+        <f t="shared" si="0"/>
         <v>184</v>
       </c>
       <c r="N2" s="10">
-        <f>SUBTOTAL(3,N4:N263)</f>
+        <f t="shared" si="0"/>
         <v>258</v>
       </c>
       <c r="O2" s="10">
-        <f>SUBTOTAL(3,O4:O263)</f>
+        <f t="shared" si="0"/>
         <v>185</v>
       </c>
       <c r="P2" s="10">
-        <f>SUBTOTAL(3,P4:P263)</f>
+        <f t="shared" si="0"/>
         <v>185</v>
       </c>
       <c r="Q2" s="10">
-        <f>SUBTOTAL(3,Q4:Q263)</f>
+        <f t="shared" si="0"/>
         <v>185</v>
       </c>
       <c r="R2" s="10">
-        <f>SUBTOTAL(3,R4:R263)</f>
+        <f t="shared" si="0"/>
         <v>185</v>
       </c>
       <c r="S2" s="10">
-        <f>SUBTOTAL(3,S4:S263)</f>
+        <f t="shared" si="0"/>
         <v>178</v>
       </c>
       <c r="T2" s="10">
-        <f>SUBTOTAL(3,T4:T263)</f>
+        <f t="shared" si="0"/>
         <v>258</v>
       </c>
       <c r="U2" s="12">
@@ -7551,78 +7551,78 @@
         <v>140</v>
       </c>
       <c r="AB2" s="12">
-        <f>SUBTOTAL(9,AB4:AB263)</f>
+        <f t="shared" ref="AB2:AI2" si="1">SUBTOTAL(9,AB4:AB263)</f>
         <v>3806212.4</v>
       </c>
       <c r="AC2" s="12">
-        <f>SUBTOTAL(9,AC4:AC263)</f>
+        <f t="shared" si="1"/>
         <v>2412673.0199999991</v>
       </c>
       <c r="AD2" s="12">
-        <f>SUBTOTAL(9,AD4:AD263)</f>
+        <f t="shared" si="1"/>
         <v>434991.12</v>
       </c>
       <c r="AE2" s="12">
-        <f>SUBTOTAL(9,AE4:AE263)</f>
+        <f t="shared" si="1"/>
         <v>415491.12</v>
       </c>
       <c r="AF2" s="12">
-        <f>SUBTOTAL(9,AF4:AF263)</f>
+        <f t="shared" si="1"/>
         <v>19500</v>
       </c>
       <c r="AG2" s="12">
-        <f>SUBTOTAL(9,AG4:AG263)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AH2" s="12">
-        <f>SUBTOTAL(9,AH4:AH263)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AI2" s="12">
-        <f>SUBTOTAL(9,AI4:AI263)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AJ2" s="10">
         <v>164</v>
       </c>
       <c r="AK2" s="12">
-        <f>SUBTOTAL(9,AK4:AK263)</f>
+        <f t="shared" ref="AK2:AT2" si="2">SUBTOTAL(9,AK4:AK263)</f>
         <v>793</v>
       </c>
       <c r="AL2" s="12">
-        <f>SUBTOTAL(9,AL4:AL263)</f>
+        <f t="shared" si="2"/>
         <v>1836733.4</v>
       </c>
       <c r="AM2" s="12">
-        <f>SUBTOTAL(9,AM4:AM263)</f>
+        <f t="shared" si="2"/>
         <v>1202031.1199999987</v>
       </c>
       <c r="AN2" s="12">
-        <f>SUBTOTAL(9,AN4:AN263)</f>
+        <f t="shared" si="2"/>
         <v>206061.59999999995</v>
       </c>
       <c r="AO2" s="12">
-        <f>SUBTOTAL(9,AO4:AO263)</f>
+        <f t="shared" si="2"/>
         <v>1408092.7199999988</v>
       </c>
       <c r="AP2" s="12">
-        <f>SUBTOTAL(9,AP4:AP263)</f>
+        <f t="shared" si="2"/>
         <v>294166.30000000005</v>
       </c>
       <c r="AQ2" s="12">
-        <f>SUBTOTAL(9,AQ4:AQ263)</f>
+        <f t="shared" si="2"/>
         <v>283738.5</v>
       </c>
       <c r="AR2" s="12">
-        <f>SUBTOTAL(9,AR4:AR263)</f>
+        <f t="shared" si="2"/>
         <v>1071665.9199999988</v>
       </c>
       <c r="AS2" s="12">
-        <f>SUBTOTAL(9,AS4:AS263)</f>
+        <f t="shared" si="2"/>
         <v>275714.5</v>
       </c>
       <c r="AT2" s="12">
-        <f>SUBTOTAL(9,AT4:AT263)</f>
+        <f t="shared" si="2"/>
         <v>188501.90000000002</v>
       </c>
       <c r="AU2" s="10">
@@ -7673,8 +7673,14 @@
       </c>
       <c r="BL2" s="10"/>
       <c r="BM2" s="10"/>
-      <c r="BN2" s="10"/>
-      <c r="BO2" s="10"/>
+      <c r="BN2" s="12">
+        <f>SUBTOTAL(9,BN4:BN263)</f>
+        <v>1750026.4199999981</v>
+      </c>
+      <c r="BO2" s="12">
+        <f>SUBTOTAL(9,BO4:BO263)</f>
+        <v>2122513.14</v>
+      </c>
     </row>
     <row r="3" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
@@ -8076,7 +8082,7 @@
         <v>0</v>
       </c>
       <c r="BP4" t="str">
-        <f t="shared" ref="BP4:BP67" si="0">G4&amp;BG4</f>
+        <f t="shared" ref="BP4:BP67" si="3">G4&amp;BG4</f>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -8277,7 +8283,7 @@
         <v>0</v>
       </c>
       <c r="BP5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -8478,7 +8484,7 @@
         <v>0</v>
       </c>
       <c r="BP6" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -8679,7 +8685,7 @@
         <v>0</v>
       </c>
       <c r="BP7" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -8880,7 +8886,7 @@
         <v>0</v>
       </c>
       <c r="BP8" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -9081,7 +9087,7 @@
         <v>4652</v>
       </c>
       <c r="BP9" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -9282,7 +9288,7 @@
         <v>0</v>
       </c>
       <c r="BP10" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -9483,7 +9489,7 @@
         <v>0</v>
       </c>
       <c r="BP11" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -9684,7 +9690,7 @@
         <v>0</v>
       </c>
       <c r="BP12" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -9885,7 +9891,7 @@
         <v>0</v>
       </c>
       <c r="BP13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -10086,7 +10092,7 @@
         <v>0</v>
       </c>
       <c r="BP14" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -10287,7 +10293,7 @@
         <v>0</v>
       </c>
       <c r="BP15" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -10488,7 +10494,7 @@
         <v>0</v>
       </c>
       <c r="BP16" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -10689,7 +10695,7 @@
         <v>0</v>
       </c>
       <c r="BP17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -10890,7 +10896,7 @@
         <v>0</v>
       </c>
       <c r="BP18" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -11091,7 +11097,7 @@
         <v>24825</v>
       </c>
       <c r="BP19" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -11288,7 +11294,7 @@
         <v>394</v>
       </c>
       <c r="BP20" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -11485,7 +11491,7 @@
         <v>394</v>
       </c>
       <c r="BP21" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -11682,7 +11688,7 @@
         <v>394</v>
       </c>
       <c r="BP22" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -11879,7 +11885,7 @@
         <v>394</v>
       </c>
       <c r="BP23" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -12080,7 +12086,7 @@
         <v>0</v>
       </c>
       <c r="BP24" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -12281,7 +12287,7 @@
         <v>0</v>
       </c>
       <c r="BP25" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -12482,7 +12488,7 @@
         <v>0</v>
       </c>
       <c r="BP26" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -12683,7 +12689,7 @@
         <v>0</v>
       </c>
       <c r="BP27" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -12884,7 +12890,7 @@
         <v>0</v>
       </c>
       <c r="BP28" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -13085,7 +13091,7 @@
         <v>0</v>
       </c>
       <c r="BP29" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -13286,7 +13292,7 @@
         <v>0</v>
       </c>
       <c r="BP30" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -13487,7 +13493,7 @@
         <v>0</v>
       </c>
       <c r="BP31" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -13688,7 +13694,7 @@
         <v>0</v>
       </c>
       <c r="BP32" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -13889,7 +13895,7 @@
         <v>0</v>
       </c>
       <c r="BP33" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -14090,7 +14096,7 @@
         <v>0</v>
       </c>
       <c r="BP34" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -14291,7 +14297,7 @@
         <v>0</v>
       </c>
       <c r="BP35" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -14492,7 +14498,7 @@
         <v>528</v>
       </c>
       <c r="BP36" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -14693,7 +14699,7 @@
         <v>0</v>
       </c>
       <c r="BP37" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -14894,7 +14900,7 @@
         <v>0</v>
       </c>
       <c r="BP38" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -15091,7 +15097,7 @@
         <v>394</v>
       </c>
       <c r="BP39" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -15292,7 +15298,7 @@
         <v>0</v>
       </c>
       <c r="BP40" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -15489,7 +15495,7 @@
         <v>394</v>
       </c>
       <c r="BP41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -15686,7 +15692,7 @@
         <v>394</v>
       </c>
       <c r="BP42" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -15887,7 +15893,7 @@
         <v>0</v>
       </c>
       <c r="BP43" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -16088,7 +16094,7 @@
         <v>0</v>
       </c>
       <c r="BP44" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -16289,7 +16295,7 @@
         <v>0</v>
       </c>
       <c r="BP45" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -16490,7 +16496,7 @@
         <v>0</v>
       </c>
       <c r="BP46" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -16691,7 +16697,7 @@
         <v>0</v>
       </c>
       <c r="BP47" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -16892,7 +16898,7 @@
         <v>0</v>
       </c>
       <c r="BP48" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -17093,7 +17099,7 @@
         <v>0</v>
       </c>
       <c r="BP49" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -17294,7 +17300,7 @@
         <v>0</v>
       </c>
       <c r="BP50" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -17495,7 +17501,7 @@
         <v>0</v>
       </c>
       <c r="BP51" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -17696,7 +17702,7 @@
         <v>0</v>
       </c>
       <c r="BP52" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -17897,7 +17903,7 @@
         <v>0</v>
       </c>
       <c r="BP53" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -18094,7 +18100,7 @@
         <v>882.59999999999945</v>
       </c>
       <c r="BP54" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -18291,7 +18297,7 @@
         <v>394</v>
       </c>
       <c r="BP55" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -18488,7 +18494,7 @@
         <v>394</v>
       </c>
       <c r="BP56" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -18685,7 +18691,7 @@
         <v>394</v>
       </c>
       <c r="BP57" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -18882,7 +18888,7 @@
         <v>394</v>
       </c>
       <c r="BP58" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -19079,7 +19085,7 @@
         <v>394</v>
       </c>
       <c r="BP59" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -19276,7 +19282,7 @@
         <v>394</v>
       </c>
       <c r="BP60" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -19473,7 +19479,7 @@
         <v>394</v>
       </c>
       <c r="BP61" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -19670,7 +19676,7 @@
         <v>394</v>
       </c>
       <c r="BP62" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -19867,7 +19873,7 @@
         <v>394</v>
       </c>
       <c r="BP63" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -20064,7 +20070,7 @@
         <v>394</v>
       </c>
       <c r="BP64" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -20261,7 +20267,7 @@
         <v>394</v>
       </c>
       <c r="BP65" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -20458,7 +20464,7 @@
         <v>394</v>
       </c>
       <c r="BP66" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -20655,7 +20661,7 @@
         <v>394</v>
       </c>
       <c r="BP67" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -20852,7 +20858,7 @@
         <v>394</v>
       </c>
       <c r="BP68" t="str">
-        <f t="shared" ref="BP68:BP131" si="1">G68&amp;BG68</f>
+        <f t="shared" ref="BP68:BP131" si="4">G68&amp;BG68</f>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -21049,7 +21055,7 @@
         <v>394</v>
       </c>
       <c r="BP69" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -21222,7 +21228,7 @@
         <v>0</v>
       </c>
       <c r="BP70" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TREDISMANTLE</v>
       </c>
     </row>
@@ -21423,7 +21429,7 @@
         <v>0</v>
       </c>
       <c r="BP71" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -21624,7 +21630,7 @@
         <v>0</v>
       </c>
       <c r="BP72" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -21825,7 +21831,7 @@
         <v>0</v>
       </c>
       <c r="BP73" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -22022,7 +22028,7 @@
         <v>394</v>
       </c>
       <c r="BP74" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -22219,7 +22225,7 @@
         <v>394</v>
       </c>
       <c r="BP75" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -22416,7 +22422,7 @@
         <v>394</v>
       </c>
       <c r="BP76" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -22613,7 +22619,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP77" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -22810,7 +22816,7 @@
         <v>942.23999999999978</v>
       </c>
       <c r="BP78" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -23007,7 +23013,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP79" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -23204,7 +23210,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP80" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -23401,7 +23407,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP81" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -23598,7 +23604,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP82" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -23795,7 +23801,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP83" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -23992,7 +23998,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP84" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -24189,7 +24195,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP85" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -24386,7 +24392,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP86" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -24583,7 +24589,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP87" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -24780,7 +24786,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP88" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -24977,7 +24983,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP89" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -25174,7 +25180,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP90" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -25371,7 +25377,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP91" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -25558,7 +25564,7 @@
         <v>0</v>
       </c>
       <c r="BP92" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>HAECANCEL</v>
       </c>
     </row>
@@ -25755,7 +25761,7 @@
         <v>882.59999999999945</v>
       </c>
       <c r="BP93" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -25952,7 +25958,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP94" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -26149,7 +26155,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP95" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -26346,7 +26352,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP96" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -26543,7 +26549,7 @@
         <v>282.59999999999991</v>
       </c>
       <c r="BP97" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -26740,7 +26746,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP98" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -26937,7 +26943,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP99" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -27134,7 +27140,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP100" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -27331,7 +27337,7 @@
         <v>394</v>
       </c>
       <c r="BP101" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -27528,7 +27534,7 @@
         <v>0</v>
       </c>
       <c r="BP102" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -27725,7 +27731,7 @@
         <v>394</v>
       </c>
       <c r="BP103" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -27922,7 +27928,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP104" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -28107,7 +28113,7 @@
         <v>0</v>
       </c>
       <c r="BP105" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMECANCEL</v>
       </c>
     </row>
@@ -28300,7 +28306,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP106" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -28501,7 +28507,7 @@
         <v>0</v>
       </c>
       <c r="BP107" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -28702,7 +28708,7 @@
         <v>0</v>
       </c>
       <c r="BP108" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -28903,7 +28909,7 @@
         <v>0</v>
       </c>
       <c r="BP109" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -29096,7 +29102,7 @@
         <v>282.59999999999991</v>
       </c>
       <c r="BP110" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -29293,7 +29299,7 @@
         <v>486.39999999999964</v>
       </c>
       <c r="BP111" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -29490,7 +29496,7 @@
         <v>0</v>
       </c>
       <c r="BP112" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -29683,7 +29689,7 @@
         <v>380.39999999999986</v>
       </c>
       <c r="BP113" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -29880,7 +29886,7 @@
         <v>380.39999999999986</v>
       </c>
       <c r="BP114" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -30077,7 +30083,7 @@
         <v>760.79999999999973</v>
       </c>
       <c r="BP115" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -30248,7 +30254,7 @@
         <v>0</v>
       </c>
       <c r="BP116" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -30419,7 +30425,7 @@
         <v>0</v>
       </c>
       <c r="BP117" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -30612,7 +30618,7 @@
         <v>882.59999999999945</v>
       </c>
       <c r="BP118" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -30813,7 +30819,7 @@
         <v>0</v>
       </c>
       <c r="BP119" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -31010,7 +31016,7 @@
         <v>282.59999999999991</v>
       </c>
       <c r="BP120" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -31211,7 +31217,7 @@
         <v>1322</v>
       </c>
       <c r="BP121" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -31412,7 +31418,7 @@
         <v>0</v>
       </c>
       <c r="BP122" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -31609,7 +31615,7 @@
         <v>394</v>
       </c>
       <c r="BP123" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -31804,7 +31810,7 @@
         <v>0</v>
       </c>
       <c r="BP124" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEIPRAN</v>
       </c>
     </row>
@@ -32005,7 +32011,7 @@
         <v>4319</v>
       </c>
       <c r="BP125" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -32206,7 +32212,7 @@
         <v>4319</v>
       </c>
       <c r="BP126" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -32395,7 +32401,7 @@
         <v>19506</v>
       </c>
       <c r="BP127" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>TMEMBB</v>
       </c>
     </row>
@@ -32592,7 +32598,7 @@
         <v>7925.4000000000015</v>
       </c>
       <c r="BP128" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -32793,7 +32799,7 @@
         <v>0</v>
       </c>
       <c r="BP129" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -32992,7 +32998,7 @@
         <v>0</v>
       </c>
       <c r="BP130" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -33193,7 +33199,7 @@
         <v>0</v>
       </c>
       <c r="BP131" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -33394,7 +33400,7 @@
         <v>0</v>
       </c>
       <c r="BP132" t="str">
-        <f t="shared" ref="BP132:BP195" si="2">G132&amp;BG132</f>
+        <f t="shared" ref="BP132:BP195" si="5">G132&amp;BG132</f>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -33593,7 +33599,7 @@
         <v>0</v>
       </c>
       <c r="BP133" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -33792,7 +33798,7 @@
         <v>0</v>
       </c>
       <c r="BP134" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -33993,7 +33999,7 @@
         <v>0</v>
       </c>
       <c r="BP135" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -34194,7 +34200,7 @@
         <v>0</v>
       </c>
       <c r="BP136" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -34393,7 +34399,7 @@
         <v>0</v>
       </c>
       <c r="BP137" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -34592,7 +34598,7 @@
         <v>0</v>
       </c>
       <c r="BP138" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -34783,7 +34789,7 @@
         <v>22904</v>
       </c>
       <c r="BP139" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -34982,7 +34988,7 @@
         <v>0</v>
       </c>
       <c r="BP140" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -35141,7 +35147,7 @@
         <v>28044</v>
       </c>
       <c r="BP141" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -35290,7 +35296,7 @@
         <v>23217</v>
       </c>
       <c r="BP142" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -35433,7 +35439,7 @@
         <v>20516</v>
       </c>
       <c r="BP143" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -35632,7 +35638,7 @@
         <v>5488.4000000000015</v>
       </c>
       <c r="BP144" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -35831,7 +35837,7 @@
         <v>0</v>
       </c>
       <c r="BP145" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -36032,7 +36038,7 @@
         <v>6335.5999999999985</v>
       </c>
       <c r="BP146" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -36175,7 +36181,7 @@
         <v>13076</v>
       </c>
       <c r="BP147" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -36318,7 +36324,7 @@
         <v>27685</v>
       </c>
       <c r="BP148" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -36515,7 +36521,7 @@
         <v>0</v>
       </c>
       <c r="BP149" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -36708,7 +36714,7 @@
         <v>4036.2000000000007</v>
       </c>
       <c r="BP150" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -36909,7 +36915,7 @@
         <v>3656</v>
       </c>
       <c r="BP151" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -37062,7 +37068,7 @@
         <v>13076</v>
       </c>
       <c r="BP152" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -37221,7 +37227,7 @@
         <v>15664</v>
       </c>
       <c r="BP153" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -37360,9 +37366,7 @@
         <v>0</v>
       </c>
       <c r="BL154" s="44"/>
-      <c r="BM154" s="36">
-        <v>-46214</v>
-      </c>
+      <c r="BM154" s="36"/>
       <c r="BN154" s="48">
         <v>0</v>
       </c>
@@ -37370,7 +37374,7 @@
         <v>12814</v>
       </c>
       <c r="BP154" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -37569,7 +37573,7 @@
         <v>0</v>
       </c>
       <c r="BP155" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -37712,7 +37716,7 @@
         <v>30319</v>
       </c>
       <c r="BP156" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -37873,7 +37877,7 @@
         <v>14099</v>
       </c>
       <c r="BP157" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -38016,7 +38020,7 @@
         <v>14474</v>
       </c>
       <c r="BP158" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -38169,7 +38173,7 @@
         <v>23695</v>
       </c>
       <c r="BP159" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -38320,7 +38324,7 @@
         <v>19584</v>
       </c>
       <c r="BP160" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -38463,7 +38467,7 @@
         <v>19251</v>
       </c>
       <c r="BP161" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -38602,9 +38606,7 @@
         <v>0</v>
       </c>
       <c r="BL162" s="44"/>
-      <c r="BM162" s="36">
-        <v>-46214</v>
-      </c>
+      <c r="BM162" s="36"/>
       <c r="BN162" s="48">
         <v>0</v>
       </c>
@@ -38612,7 +38614,7 @@
         <v>15664</v>
       </c>
       <c r="BP162" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -38755,7 +38757,7 @@
         <v>20395</v>
       </c>
       <c r="BP163" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -38914,7 +38916,7 @@
         <v>19507</v>
       </c>
       <c r="BP164" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -39057,7 +39059,7 @@
         <v>20395</v>
       </c>
       <c r="BP165" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -39258,7 +39260,7 @@
         <v>0</v>
       </c>
       <c r="BP166" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -39409,7 +39411,7 @@
         <v>14474</v>
       </c>
       <c r="BP167" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -39608,7 +39610,7 @@
         <v>0</v>
       </c>
       <c r="BP168" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -39767,7 +39769,7 @@
         <v>12836</v>
       </c>
       <c r="BP169" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -39910,7 +39912,7 @@
         <v>17423</v>
       </c>
       <c r="BP170" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -40065,7 +40067,7 @@
         <v>23782</v>
       </c>
       <c r="BP171" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -40266,7 +40268,7 @@
         <v>0</v>
       </c>
       <c r="BP172" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -40467,7 +40469,7 @@
         <v>2277</v>
       </c>
       <c r="BP173" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -40626,7 +40628,7 @@
         <v>13076</v>
       </c>
       <c r="BP174" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -40825,7 +40827,7 @@
         <v>0</v>
       </c>
       <c r="BP175" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -40974,7 +40976,7 @@
         <v>20362</v>
       </c>
       <c r="BP176" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -41127,7 +41129,7 @@
         <v>26066</v>
       </c>
       <c r="BP177" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -41270,7 +41272,7 @@
         <v>13076</v>
       </c>
       <c r="BP178" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -41469,7 +41471,7 @@
         <v>0</v>
       </c>
       <c r="BP179" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -41626,7 +41628,7 @@
         <v>29885</v>
       </c>
       <c r="BP180" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -41785,7 +41787,7 @@
         <v>12814</v>
       </c>
       <c r="BP181" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -41982,7 +41984,7 @@
         <v>1117.2999999999993</v>
       </c>
       <c r="BP182" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -42125,7 +42127,7 @@
         <v>17547</v>
       </c>
       <c r="BP183" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -42268,7 +42270,7 @@
         <v>14749</v>
       </c>
       <c r="BP184" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -42411,7 +42413,7 @@
         <v>14749</v>
       </c>
       <c r="BP185" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -42554,7 +42556,7 @@
         <v>14749</v>
       </c>
       <c r="BP186" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -42697,7 +42699,7 @@
         <v>14749</v>
       </c>
       <c r="BP187" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -42840,7 +42842,7 @@
         <v>14749</v>
       </c>
       <c r="BP188" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -42983,7 +42985,7 @@
         <v>14749</v>
       </c>
       <c r="BP189" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -43126,7 +43128,7 @@
         <v>14749</v>
       </c>
       <c r="BP190" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -43269,7 +43271,7 @@
         <v>14749</v>
       </c>
       <c r="BP191" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -43462,7 +43464,7 @@
         <v>3547.1000000000004</v>
       </c>
       <c r="BP192" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -43659,7 +43661,7 @@
         <v>0</v>
       </c>
       <c r="BP193" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -43852,7 +43854,7 @@
         <v>3259.5</v>
       </c>
       <c r="BP194" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -44013,7 +44015,7 @@
         <v>17661</v>
       </c>
       <c r="BP195" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -44206,7 +44208,7 @@
         <v>4166.7000000000007</v>
       </c>
       <c r="BP196" t="str">
-        <f t="shared" ref="BP196:BP263" si="3">G196&amp;BG196</f>
+        <f t="shared" ref="BP196:BP263" si="6">G196&amp;BG196</f>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -44349,7 +44351,7 @@
         <v>21150</v>
       </c>
       <c r="BP197" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -44492,7 +44494,7 @@
         <v>17566</v>
       </c>
       <c r="BP198" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -44687,7 +44689,7 @@
         <v>25150.5</v>
       </c>
       <c r="BP199" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -44882,7 +44884,7 @@
         <v>4842.6000000000004</v>
       </c>
       <c r="BP200" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -45025,7 +45027,7 @@
         <v>17566</v>
       </c>
       <c r="BP201" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -45168,7 +45170,7 @@
         <v>21139</v>
       </c>
       <c r="BP202" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -45311,7 +45313,7 @@
         <v>21150</v>
       </c>
       <c r="BP203" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -45506,7 +45508,7 @@
         <v>4328.1000000000022</v>
       </c>
       <c r="BP204" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -45699,7 +45701,7 @@
         <v>5907</v>
       </c>
       <c r="BP205" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -45842,7 +45844,7 @@
         <v>24723</v>
       </c>
       <c r="BP206" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -46037,7 +46039,7 @@
         <v>5108.1000000000022</v>
       </c>
       <c r="BP207" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -46180,7 +46182,7 @@
         <v>17566</v>
       </c>
       <c r="BP208" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -46323,7 +46325,7 @@
         <v>26766</v>
       </c>
       <c r="BP209" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -46518,7 +46520,7 @@
         <v>6967.7999999999993</v>
       </c>
       <c r="BP210" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -46661,7 +46663,7 @@
         <v>17566</v>
       </c>
       <c r="BP211" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -46858,7 +46860,7 @@
         <v>5578.0999999999985</v>
       </c>
       <c r="BP212" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -47051,7 +47053,7 @@
         <v>4869</v>
       </c>
       <c r="BP213" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -47196,7 +47198,7 @@
         <v>30863</v>
       </c>
       <c r="BP214" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>TMEMBB</v>
       </c>
     </row>
@@ -47339,7 +47341,7 @@
         <v>5107</v>
       </c>
       <c r="BP215" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>TMEBATERRY</v>
       </c>
     </row>
@@ -47534,7 +47536,7 @@
         <v>11188.300000000001</v>
       </c>
       <c r="BP216" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>TMEMBB</v>
       </c>
     </row>
@@ -47689,7 +47691,7 @@
         <v>25971</v>
       </c>
       <c r="BP217" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>TMEMBB</v>
       </c>
     </row>
@@ -47832,7 +47834,7 @@
         <v>3474</v>
       </c>
       <c r="BP218" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>TMEMBB</v>
       </c>
     </row>
@@ -47993,7 +47995,7 @@
         <v>27088</v>
       </c>
       <c r="BP219" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>TMEMBB</v>
       </c>
     </row>
@@ -48136,7 +48138,7 @@
         <v>13732</v>
       </c>
       <c r="BP220" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -48279,7 +48281,7 @@
         <v>22854</v>
       </c>
       <c r="BP221" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -48422,7 +48424,7 @@
         <v>28459</v>
       </c>
       <c r="BP222" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -48565,7 +48567,7 @@
         <v>16954</v>
       </c>
       <c r="BP223" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -48708,7 +48710,7 @@
         <v>21663</v>
       </c>
       <c r="BP224" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -48851,7 +48853,7 @@
         <v>19904</v>
       </c>
       <c r="BP225" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -48994,7 +48996,7 @@
         <v>18746</v>
       </c>
       <c r="BP226" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -49137,7 +49139,7 @@
         <v>16954</v>
       </c>
       <c r="BP227" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -49280,7 +49282,7 @@
         <v>15785</v>
       </c>
       <c r="BP228" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -49423,7 +49425,7 @@
         <v>26187</v>
       </c>
       <c r="BP229" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -49566,7 +49568,7 @@
         <v>22854</v>
       </c>
       <c r="BP230" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -49709,7 +49711,7 @@
         <v>22854</v>
       </c>
       <c r="BP231" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -49852,7 +49854,7 @@
         <v>13994</v>
       </c>
       <c r="BP232" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -49995,7 +49997,7 @@
         <v>22854</v>
       </c>
       <c r="BP233" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -50138,7 +50140,7 @@
         <v>17065</v>
       </c>
       <c r="BP234" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -50281,7 +50283,7 @@
         <v>14890</v>
       </c>
       <c r="BP235" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -50424,7 +50426,7 @@
         <v>22220</v>
       </c>
       <c r="BP236" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -50567,7 +50569,7 @@
         <v>25007</v>
       </c>
       <c r="BP237" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -50710,7 +50712,7 @@
         <v>12574</v>
       </c>
       <c r="BP238" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -50853,7 +50855,7 @@
         <v>23444</v>
       </c>
       <c r="BP239" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -50996,7 +50998,7 @@
         <v>22854</v>
       </c>
       <c r="BP240" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -51139,7 +51141,7 @@
         <v>22088</v>
       </c>
       <c r="BP241" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -51282,7 +51284,7 @@
         <v>18223</v>
       </c>
       <c r="BP242" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -51425,7 +51427,7 @@
         <v>22854</v>
       </c>
       <c r="BP243" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -51568,7 +51570,7 @@
         <v>19882</v>
       </c>
       <c r="BP244" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -51711,7 +51713,7 @@
         <v>18839</v>
       </c>
       <c r="BP245" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -51854,7 +51856,7 @@
         <v>13732</v>
       </c>
       <c r="BP246" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -51997,7 +51999,7 @@
         <v>17566</v>
       </c>
       <c r="BP247" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -52140,7 +52142,7 @@
         <v>22854</v>
       </c>
       <c r="BP248" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -52283,7 +52285,7 @@
         <v>27925</v>
       </c>
       <c r="BP249" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -52426,7 +52428,7 @@
         <v>19358</v>
       </c>
       <c r="BP250" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -52569,7 +52571,7 @@
         <v>25321</v>
       </c>
       <c r="BP251" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -52712,7 +52714,7 @@
         <v>18112</v>
       </c>
       <c r="BP252" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -52855,7 +52857,7 @@
         <v>26187</v>
       </c>
       <c r="BP253" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -52998,7 +53000,7 @@
         <v>18112</v>
       </c>
       <c r="BP254" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -53141,7 +53143,7 @@
         <v>22854</v>
       </c>
       <c r="BP255" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -53284,7 +53286,7 @@
         <v>27102</v>
       </c>
       <c r="BP256" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -53427,7 +53429,7 @@
         <v>19904</v>
       </c>
       <c r="BP257" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -53570,7 +53572,7 @@
         <v>23551</v>
       </c>
       <c r="BP258" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -53713,7 +53715,7 @@
         <v>20513</v>
       </c>
       <c r="BP259" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>HAEMBB</v>
       </c>
     </row>
@@ -53848,7 +53850,7 @@
         <v>21822</v>
       </c>
       <c r="BP260" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>TMEMBB</v>
       </c>
     </row>
@@ -53979,7 +53981,7 @@
         <v>21563</v>
       </c>
       <c r="BP261" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>TMEMBB</v>
       </c>
     </row>
@@ -54110,7 +54112,7 @@
         <v>21229</v>
       </c>
       <c r="BP262" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>TMEMBB</v>
       </c>
     </row>
@@ -54245,7 +54247,7 @@
         <v>32571</v>
       </c>
       <c r="BP263" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>TMEMBB</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: align template and JS parsing - NaN days, WK- slots, AC1/AC2 breakdown
</commit_message>
<xml_diff>
--- a/Dashboard_Template_30_Slides_Final.xlsx
+++ b/Dashboard_Template_30_Slides_Final.xlsx
@@ -431,7 +431,7 @@
       <c r="C2" t="str">
         <v>Report Week</v>
       </c>
-      <c r="D2" t="str">
+      <c r="D2">
         <v>26</v>
       </c>
       <c r="E2" t="str">
@@ -448,8 +448,8 @@
       <c r="C3" t="str">
         <v>HAE M1 Avg</v>
       </c>
-      <c r="D3" t="str">
-        <v>365.56 วัน</v>
+      <c r="D3">
+        <v>365.56</v>
       </c>
       <c r="E3" t="str">
         <v>หน้างานยังคงเดินหน้าอย่างรวดเร็ว แต่ระบบเอกสารยังมีปัญหาคอขวด</v>
@@ -465,8 +465,8 @@
       <c r="C4" t="str">
         <v>TME M1 Avg</v>
       </c>
-      <c r="D4" t="str">
-        <v>-542.98 วัน</v>
+      <c r="D4">
+        <v>-542.98</v>
       </c>
       <c r="E4" t="str">
         <v>ข้อมูลดิบอาจมีความคลาดเคลื่อนในระบบ</v>
@@ -549,7 +549,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:G11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -568,6 +568,9 @@
         <v>M2 Aging</v>
       </c>
       <c r="F1" t="str">
+        <v>Sites</v>
+      </c>
+      <c r="G1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -588,6 +591,9 @@
         <v/>
       </c>
       <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
         <v>หน้างานทำได้เร็ว แต่กระบวนการตรวจรับเอกสารล่าช้า</v>
       </c>
     </row>
@@ -599,16 +605,19 @@
         <v>1st Milestone AGING Analysis</v>
       </c>
       <c r="C3" t="str">
-        <v>HAE</v>
-      </c>
-      <c r="D3" t="str">
+        <v>HAE M1</v>
+      </c>
+      <c r="D3">
         <v>365.56</v>
       </c>
       <c r="E3" t="str">
         <v/>
       </c>
-      <c r="F3" t="str">
-        <v>เปรียบเทียบระยะเวลาปิด M1</v>
+      <c r="F3">
+        <v>169</v>
+      </c>
+      <c r="G3" t="str">
+        <v>เปรียบเทียบระยะเวลาปิด M1 สำหรับ HAE</v>
       </c>
     </row>
     <row r="4">
@@ -619,16 +628,19 @@
         <v>1st Milestone AGING Analysis</v>
       </c>
       <c r="C4" t="str">
-        <v>TME</v>
-      </c>
-      <c r="D4" t="str">
-        <v/>
+        <v>TME M1</v>
+      </c>
+      <c r="D4">
+        <v>-542.98</v>
       </c>
       <c r="E4" t="str">
         <v/>
       </c>
-      <c r="F4" t="str">
-        <v>เปรียบเทียบระยะเวลาปิด M1</v>
+      <c r="F4">
+        <v>87</v>
+      </c>
+      <c r="G4" t="str">
+        <v>เปรียบเทียบระยะเวลาปิด M1 สำหรับ TME</v>
       </c>
     </row>
     <row r="5">
@@ -639,81 +651,162 @@
         <v>2nd Milestone AGING Analysis</v>
       </c>
       <c r="C5" t="str">
-        <v>Overall M2</v>
+        <v>HAE M2</v>
       </c>
       <c r="D5" t="str">
         <v/>
       </c>
-      <c r="E5" t="str">
-        <v/>
+      <c r="E5">
+        <v>18</v>
       </c>
       <c r="F5" t="str">
-        <v>ความท้าทายในการปิดเอกสาร M2 ที่กินระยะเวลานาน</v>
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>HAE M2 Avg Aging</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Slide 10</v>
+        <v>Slide 9</v>
       </c>
       <c r="B6" t="str">
-        <v>Performance by PE Owner: Adisak</v>
+        <v>2nd Milestone AGING Analysis</v>
       </c>
       <c r="C6" t="str">
-        <v>Adisak Chanmao</v>
+        <v>TME M2 MBB</v>
       </c>
       <c r="D6" t="str">
-        <v>1.83</v>
-      </c>
-      <c r="E6" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="E6">
+        <v>3</v>
       </c>
       <c r="F6" t="str">
-        <v>ชื่นชมความรวดเร็วใน M1 แต่เน้นย้ำให้ช่วยผลักดัน M2</v>
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v>TME M2 MBB Avg Aging</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Slide 11</v>
+        <v>Slide 10</v>
       </c>
       <c r="B7" t="str">
-        <v>Performance by PE Owner: Palagon</v>
+        <v>Performance by PE Owner: Adisak</v>
       </c>
       <c r="C7" t="str">
-        <v>Palagon Prommueangma</v>
-      </c>
-      <c r="D7" t="str">
-        <v/>
+        <v>Adisak Chanmao Average</v>
+      </c>
+      <c r="D7">
+        <v>1.83</v>
       </c>
       <c r="E7" t="str">
         <v/>
       </c>
-      <c r="F7" t="str">
-        <v>เปรียบเทียบเทคนิคการทำงานเพื่อหา Best Practice</v>
+      <c r="F7">
+        <v>87</v>
+      </c>
+      <c r="G7" t="str">
+        <v>ชื่นชมความรวดเร็วใน M1 แต่เน้นย้ำให้ช่วยผลักดัน M2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>Slide 11</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Performance by PE Owner: Palagon</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Palagon Prommueangma Average</v>
+      </c>
+      <c r="D8">
+        <v>3.57</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8">
+        <v>169</v>
+      </c>
+      <c r="G8" t="str">
+        <v>เปรียบเทียบเทคนิคการทำงานเพื่อหา Best Practice</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Slide 11</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Performance by PE Owner: Palagon</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Palagon HAE</v>
+      </c>
+      <c r="D9">
+        <v>3.57</v>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v>Palagon HAE M1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Slide 11</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Performance by PE Owner: Palagon</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Palagon TME</v>
+      </c>
+      <c r="D10">
+        <v>2.5</v>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v>Palagon TME M1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>Slide 12</v>
       </c>
-      <c r="B8" t="str">
+      <c r="B11" t="str">
         <v>PE Performance Comparison</v>
       </c>
-      <c r="C8" t="str">
+      <c r="C11" t="str">
         <v>Watch-list</v>
       </c>
-      <c r="D8" t="str">
-        <v/>
-      </c>
-      <c r="E8" t="str">
-        <v/>
-      </c>
-      <c r="F8" t="str">
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
         <v>สรุปภาพรวมและจัดทำ Watch-list ของไซต์ที่เกิน SLA</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -756,7 +849,7 @@
         <v>Slide 13</v>
       </c>
       <c r="B2" t="str">
-        <v>Document Owner Performance</v>
+        <v>Acceptance Performance</v>
       </c>
       <c r="C2" t="str">
         <v>AC#1 (JAN-DEC)</v>
@@ -764,20 +857,20 @@
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
+      <c r="E2">
         <v>1510000</v>
       </c>
       <c r="F2" t="str">
         <v/>
       </c>
-      <c r="G2" t="str">
+      <c r="G2">
         <v>8290000</v>
       </c>
-      <c r="H2" t="str">
-        <v/>
+      <c r="H2">
+        <v>15.5</v>
       </c>
       <c r="I2" t="str">
-        <v>AC#1 Total Amount / Done</v>
+        <v>AC#1 Total — Avg Aging ใส่ค่าตัวเลข เช่น 15.5</v>
       </c>
     </row>
     <row r="3">
@@ -785,7 +878,7 @@
         <v>Slide 13</v>
       </c>
       <c r="B3" t="str">
-        <v>Document Owner Performance</v>
+        <v>Acceptance Performance</v>
       </c>
       <c r="C3" t="str">
         <v>AC#2 (JAN-DEC)</v>
@@ -793,20 +886,20 @@
       <c r="D3" t="str">
         <v/>
       </c>
-      <c r="E3" t="str">
+      <c r="E3">
         <v>349000</v>
       </c>
       <c r="F3" t="str">
         <v/>
       </c>
-      <c r="G3" t="str">
+      <c r="G3">
         <v>4700000</v>
       </c>
-      <c r="H3" t="str">
-        <v/>
+      <c r="H3">
+        <v>33</v>
       </c>
       <c r="I3" t="str">
-        <v>AC#2 Total Amount / Done</v>
+        <v>AC#2 Total — Avg Aging ใส่ค่าตัวเลข</v>
       </c>
     </row>
     <row r="4">
@@ -819,10 +912,10 @@
       <c r="C4" t="str">
         <v>Hathairat AC1</v>
       </c>
-      <c r="D4" t="str">
+      <c r="D4">
         <v>41</v>
       </c>
-      <c r="E4" t="str">
+      <c r="E4">
         <v>693559</v>
       </c>
       <c r="F4" t="str">
@@ -831,11 +924,11 @@
       <c r="G4" t="str">
         <v/>
       </c>
-      <c r="H4" t="str">
-        <v/>
+      <c r="H4">
+        <v>15.98</v>
       </c>
       <c r="I4" t="str">
-        <v>AC#1 Aging สำหรับ น.ส.หทัยรัตน์</v>
+        <v>AC#1 Avg Aging สำหรับ น.ส.หทัยรัตน์ (ตัวเลขเท่านั้น)</v>
       </c>
     </row>
     <row r="5">
@@ -854,17 +947,17 @@
       <c r="E5" t="str">
         <v/>
       </c>
-      <c r="F5" t="str">
-        <v>0</v>
+      <c r="F5">
+        <v>50000</v>
       </c>
       <c r="G5" t="str">
         <v/>
       </c>
-      <c r="H5" t="str">
-        <v/>
+      <c r="H5">
+        <v>33.15</v>
       </c>
       <c r="I5" t="str">
-        <v>AC#2 Aging / Amount สำหรับ น.ส.หทัยรัตน์</v>
+        <v>AC#2 Avg Aging + AC2 Amount สำหรับ น.ส.หทัยรัตน์</v>
       </c>
     </row>
     <row r="6">
@@ -877,10 +970,10 @@
       <c r="C6" t="str">
         <v>Sermsiri AC1</v>
       </c>
-      <c r="D6" t="str">
+      <c r="D6">
         <v>50</v>
       </c>
-      <c r="E6" t="str">
+      <c r="E6">
         <v>113164</v>
       </c>
       <c r="F6" t="str">
@@ -889,11 +982,11 @@
       <c r="G6" t="str">
         <v/>
       </c>
-      <c r="H6" t="str">
-        <v/>
+      <c r="H6">
+        <v>15.46</v>
       </c>
       <c r="I6" t="str">
-        <v>AC#1 Aging สำหรับ Sermsiri (IPRAN/TME)</v>
+        <v>AC#1 Avg Aging สำหรับ Sermsiri (ตัวเลขเท่านั้น)</v>
       </c>
     </row>
     <row r="7">
@@ -912,17 +1005,17 @@
       <c r="E7" t="str">
         <v/>
       </c>
-      <c r="F7" t="str">
-        <v>0</v>
+      <c r="F7">
+        <v>30000</v>
       </c>
       <c r="G7" t="str">
         <v/>
       </c>
-      <c r="H7" t="str">
-        <v/>
+      <c r="H7">
+        <v>49</v>
       </c>
       <c r="I7" t="str">
-        <v>AC#2 Aging / Amount สำหรับ Sermsiri</v>
+        <v>AC#2 Avg Aging + AC2 Amount สำหรับ Sermsiri</v>
       </c>
     </row>
     <row r="8">
@@ -935,10 +1028,10 @@
       <c r="C8" t="str">
         <v>Apichart AC1</v>
       </c>
-      <c r="D8" t="str">
+      <c r="D8">
         <v>26</v>
       </c>
-      <c r="E8" t="str">
+      <c r="E8">
         <v>138325</v>
       </c>
       <c r="F8" t="str">
@@ -947,11 +1040,11 @@
       <c r="G8" t="str">
         <v/>
       </c>
-      <c r="H8" t="str">
-        <v/>
+      <c r="H8">
+        <v>14.88</v>
       </c>
       <c r="I8" t="str">
-        <v>AC#1 Aging สำหรับ Apichart (MBB/HAE)</v>
+        <v>AC#1 Avg Aging สำหรับ Apichart (ตัวเลขเท่านั้น)</v>
       </c>
     </row>
     <row r="9">
@@ -970,17 +1063,17 @@
       <c r="E9" t="str">
         <v/>
       </c>
-      <c r="F9" t="str">
+      <c r="F9">
         <v>0</v>
       </c>
       <c r="G9" t="str">
         <v/>
       </c>
-      <c r="H9" t="str">
-        <v/>
+      <c r="H9">
+        <v>0</v>
       </c>
       <c r="I9" t="str">
-        <v>AC#2 Aging / Amount สำหรับ Apichart</v>
+        <v>AC#2 Avg Aging สำหรับ Apichart (0 ถ้าไม่มีข้อมูล)</v>
       </c>
     </row>
     <row r="10">
@@ -988,15 +1081,15 @@
         <v>Slide 19</v>
       </c>
       <c r="B10" t="str">
-        <v>Overall Team Install WK27</v>
+        <v>Overall Team Install</v>
       </c>
       <c r="C10" t="str">
         <v>Overall Team Install WK27</v>
       </c>
-      <c r="D10" t="str">
+      <c r="D10">
         <v>45</v>
       </c>
-      <c r="E10" t="str">
+      <c r="E10">
         <v>113101</v>
       </c>
       <c r="F10" t="str">
@@ -1005,11 +1098,11 @@
       <c r="G10" t="str">
         <v/>
       </c>
-      <c r="H10" t="str">
+      <c r="H10">
         <v>6</v>
       </c>
       <c r="I10" t="str">
-        <v>WK27: จำนวน site / Amount / Avg Aging</v>
+        <v>WK27: Sites=จำนวนไซต์, Amount=ยอดเงิน, Avg Aging=ตัวเลข</v>
       </c>
     </row>
     <row r="11">
@@ -1017,15 +1110,15 @@
         <v>Slide 19</v>
       </c>
       <c r="B11" t="str">
-        <v>Overall Team Install WK28</v>
+        <v>Overall Team Install</v>
       </c>
       <c r="C11" t="str">
         <v>Overall Team Install WK28</v>
       </c>
-      <c r="D11" t="str">
+      <c r="D11">
         <v>62</v>
       </c>
-      <c r="E11" t="str">
+      <c r="E11">
         <v>201167</v>
       </c>
       <c r="F11" t="str">
@@ -1034,11 +1127,11 @@
       <c r="G11" t="str">
         <v/>
       </c>
-      <c r="H11" t="str">
+      <c r="H11">
         <v>11</v>
       </c>
       <c r="I11" t="str">
-        <v>WK28: จำนวน site / Amount / Avg Aging</v>
+        <v>WK28: Sites=จำนวนไซต์, Amount=ยอดเงิน, Avg Aging=ตัวเลข</v>
       </c>
     </row>
     <row r="12">
@@ -1079,7 +1172,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E30"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1108,7 +1201,7 @@
       <c r="C2" t="str">
         <v>Estimate Final Income</v>
       </c>
-      <c r="D2" t="str">
+      <c r="D2">
         <v>3180000</v>
       </c>
       <c r="E2" t="str">
@@ -1125,7 +1218,7 @@
       <c r="C3" t="str">
         <v>AR (Commerce)</v>
       </c>
-      <c r="D3" t="str">
+      <c r="D3">
         <v>1730000</v>
       </c>
       <c r="E3" t="str">
@@ -1142,7 +1235,7 @@
       <c r="C4" t="str">
         <v>AP (Payment)</v>
       </c>
-      <c r="D4" t="str">
+      <c r="D4">
         <v>635000</v>
       </c>
       <c r="E4" t="str">
@@ -1159,7 +1252,7 @@
       <c r="C5" t="str">
         <v>Remain to Claim</v>
       </c>
-      <c r="D5" t="str">
+      <c r="D5">
         <v>1140000</v>
       </c>
       <c r="E5" t="str">
@@ -1176,11 +1269,11 @@
       <c r="C6" t="str">
         <v>Backlog Week 25</v>
       </c>
-      <c r="D6" t="str">
-        <v/>
+      <c r="D6">
+        <v>1500000</v>
       </c>
       <c r="E6" t="str">
-        <v>เปรียบเทียบเป้าหมายการเก็บเงินระหว่างสัปดาห์</v>
+        <v>WK25 Backlog ใส่เป็นตัวเลข</v>
       </c>
     </row>
     <row r="7">
@@ -1193,11 +1286,11 @@
       <c r="C7" t="str">
         <v>Backlog Week 26</v>
       </c>
-      <c r="D7" t="str">
-        <v/>
+      <c r="D7">
+        <v>1350000</v>
       </c>
       <c r="E7" t="str">
-        <v>กราฟเส้นแนวโน้มยอดคงค้าง</v>
+        <v>WK26 Backlog ใส่เป็นตัวเลข</v>
       </c>
     </row>
     <row r="8">
@@ -1205,72 +1298,395 @@
         <v>Slide 24</v>
       </c>
       <c r="B8" t="str">
-        <v>Recovery Plan: Acceptance Plan</v>
+        <v>Actual Acceptance</v>
       </c>
       <c r="C8" t="str">
-        <v>Target JUNE</v>
-      </c>
-      <c r="D8" t="str">
-        <v/>
+        <v>Actual Acceptance WK23</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
       </c>
       <c r="E8" t="str">
-        <v>ยอด Remain ที่ตั้งเป้าจะเคลียร์ (2023-2026)</v>
+        <v>WK23 ยอด Actual Acceptance (ตัวเลข ฿)</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Slide 25</v>
+        <v>Slide 24</v>
       </c>
       <c r="B9" t="str">
-        <v>Recovery Plan: Action Plan AC#2</v>
+        <v>Actual Acceptance</v>
       </c>
       <c r="C9" t="str">
-        <v>Action Plan AC#2</v>
-      </c>
-      <c r="D9" t="str">
-        <v/>
+        <v>Actual Acceptance WK24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
       </c>
       <c r="E9" t="str">
-        <v>แผนผลักดัน AC#2 สู่การรับรู้รายได้</v>
+        <v>WK24 ยอด Actual Acceptance (ตัวเลข ฿)</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Slide 26</v>
+        <v>Slide 24</v>
       </c>
       <c r="B10" t="str">
-        <v>Recovery Plan: Install On-Process</v>
+        <v>Actual Acceptance</v>
       </c>
       <c r="C10" t="str">
-        <v>On-Process (2026)</v>
-      </c>
-      <c r="D10" t="str">
-        <v/>
+        <v>Actual Acceptance WK25</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
       </c>
       <c r="E10" t="str">
-        <v>มูลค่างาน In-house ที่อยู่ระหว่างดำเนินการ</v>
+        <v>WK25 ยอด Actual Acceptance (ตัวเลข ฿)</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v>Slide 24</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Actual Acceptance</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Actual Acceptance WK26</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="str">
+        <v>WK26 ยอด Actual Acceptance (ตัวเลข ฿)</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Slide 24</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Actual Acceptance</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Actual Acceptance WK27</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="str">
+        <v>WK27 ยอด Actual Acceptance (ตัวเลข ฿)</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Slide 24</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Actual Acceptance Total</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Actual Acceptance July Total</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" t="str">
+        <v>JULY Total รวม (ตัวเลข ฿)</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Slide 24</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Actual Acceptance Total</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Actual Acceptance Total (JAN-JULY) HUAWEI</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14" t="str">
+        <v>HUAWEI JAN-JULY (ตัวเลข ฿)</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Slide 24</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Actual Acceptance Total</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Actual Acceptance Total (JAN-JULY) TRUE-TUC</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15" t="str">
+        <v>TRUE-TUC JAN-JULY (ตัวเลข ฿)</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Slide 25</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Acceptance AC#1 Plan (2023)</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Action Plan AC#1</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16" t="str">
+        <v>AC#1 Plan ปี 2023 (ตัวเลข ฿)</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Slide 25</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Acceptance AC#1 Plan (2024)</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Action Plan AC#1</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="str">
+        <v>AC#1 Plan ปี 2024 (ตัวเลข ฿)</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Slide 25</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Acceptance AC#1 Plan (2025)</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Action Plan AC#1</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="str">
+        <v>AC#1 Plan ปี 2025 (ตัวเลข ฿)</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Slide 25</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Acceptance AC#1 Plan (2026)</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Action Plan AC#1</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="str">
+        <v>AC#1 Plan ปี 2026 (ตัวเลข ฿)</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Slide 25</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Acceptance AC#2 Plan (2023)</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Action Plan AC#2</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20" t="str">
+        <v>AC#2 Plan ปี 2023 (ตัวเลข ฿)</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Slide 25</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Acceptance AC#2 Plan (2024)</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Action Plan AC#2</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="str">
+        <v>AC#2 Plan ปี 2024 (ตัวเลข ฿)</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Slide 25</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Acceptance AC#2 Plan (2025)</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Action Plan AC#2</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22" t="str">
+        <v>AC#2 Plan ปี 2025 (ตัวเลข ฿)</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Slide 25</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Acceptance AC#2 Plan (2026)</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Action Plan AC#2</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23" t="str">
+        <v>AC#2 Plan ปี 2026 (ตัวเลข ฿)</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Slide 26</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Install On-Process</v>
+      </c>
+      <c r="C24" t="str">
+        <v>On-Process TME-MBB</v>
+      </c>
+      <c r="D24">
+        <v>230347</v>
+      </c>
+      <c r="E24" t="str">
+        <v>TME-MBB On-Process Amount (ตัวเลข ฿)</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Slide 26</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Install On-Process</v>
+      </c>
+      <c r="C25" t="str">
+        <v>On-Process TME-IPRAN</v>
+      </c>
+      <c r="D25">
+        <v>225486</v>
+      </c>
+      <c r="E25" t="str">
+        <v>TME-IPRAN On-Process Amount</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Slide 26</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Install On-Process</v>
+      </c>
+      <c r="C26" t="str">
+        <v>On-Process TME-BATTERY</v>
+      </c>
+      <c r="D26">
+        <v>5107</v>
+      </c>
+      <c r="E26" t="str">
+        <v>TME-BATTERY On-Process Amount</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Slide 26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Install On-Process</v>
+      </c>
+      <c r="C27" t="str">
+        <v>On-Process HAE-MBB</v>
+      </c>
+      <c r="D27">
+        <v>3348098</v>
+      </c>
+      <c r="E27" t="str">
+        <v>HAE-MBB On-Process Amount</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Slide 26</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Install On-Process</v>
+      </c>
+      <c r="C28" t="str">
+        <v>On-Process TRE-DISMANTLE</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28" t="str">
+        <v>TRE-DISMANTLE On-Process Amount</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
         <v>Slide 27</v>
       </c>
-      <c r="B11" t="str">
+      <c r="B29" t="str">
+        <v>Action Plan Total</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Action Plan Total WK26</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Action Plan Total WK## ล่าสุด (ตัวเลข ฿)</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Slide 27</v>
+      </c>
+      <c r="B30" t="str">
         <v>Summary of REMAIN (3 Pillars)</v>
       </c>
-      <c r="C11" t="str">
+      <c r="C30" t="str">
         <v>AC1 DONE / UNFULFILL / Total</v>
       </c>
-      <c r="D11" t="str">
-        <v/>
-      </c>
-      <c r="E11" t="str">
+      <c r="D30" t="str">
+        <v/>
+      </c>
+      <c r="E30" t="str">
         <v>สรุปภาพรวมยอดค้าง 3 ส่วนหลัก</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E30"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix: multiple dashboard parsing issues (Huawei/True, Aging MIN, SO Compare, SLA Summary, DOC Owner AC2)
</commit_message>
<xml_diff>
--- a/Dashboard_Template_30_Slides_Final.xlsx
+++ b/Dashboard_Template_30_Slides_Final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\0_Dashboad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34E2FEFF-73B5-4D09-A6EC-A72B7F3D6743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ADDE88D-16F4-42D2-AF91-056C81D965A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="813" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="813" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Part 1 - Overview" sheetId="1" r:id="rId1"/>
@@ -4207,12 +4207,6 @@
     <t>ยอด Actual Acceptance WK27</t>
   </si>
   <si>
-    <t>ยอด Actual Actual Acceptance TOTAL (JAN-JUNE) HUAWEI</t>
-  </si>
-  <si>
-    <t>ยอด Actual Actual Acceptance TOTAL (JAN-JUNE) TRUE-TUC</t>
-  </si>
-  <si>
     <t>WEEK28</t>
   </si>
   <si>
@@ -4376,6 +4370,12 @@
   </si>
   <si>
     <t>12 วัน</t>
+  </si>
+  <si>
+    <t>ยอด Actual Actual Acceptance TOTAL (JAN-JULY) HUAWEI</t>
+  </si>
+  <si>
+    <t>ยอด Actual Actual Acceptance TOTAL (JAN-JULY) TRUE-TUC</t>
   </si>
 </sst>
 </file>
@@ -5095,6 +5095,18 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -5109,18 +5121,6 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -5506,7 +5506,7 @@
         <v>29</v>
       </c>
       <c r="E2" t="s">
-        <v>1375</v>
+        <v>1373</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -5898,10 +5898,10 @@
         <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>1377</v>
+        <v>1375</v>
       </c>
       <c r="C3" t="s">
-        <v>1377</v>
+        <v>1375</v>
       </c>
       <c r="D3">
         <v>247932</v>
@@ -5913,7 +5913,7 @@
         <v>13</v>
       </c>
       <c r="G3" t="s">
-        <v>1376</v>
+        <v>1374</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -6170,7 +6170,7 @@
         <v>55</v>
       </c>
       <c r="B6" t="s">
-        <v>1355</v>
+        <v>1353</v>
       </c>
       <c r="C6" t="s">
         <v>95</v>
@@ -6188,14 +6188,14 @@
         <v>55</v>
       </c>
       <c r="B7" t="s">
-        <v>1355</v>
+        <v>1353</v>
       </c>
       <c r="C7" t="s">
-        <v>1354</v>
+        <v>1352</v>
       </c>
       <c r="D7" s="49">
         <f>Sheet1!N20</f>
-        <v>2395760.7200000002</v>
+        <v>2317847.48</v>
       </c>
       <c r="E7" t="s">
         <v>96</v>
@@ -6246,7 +6246,7 @@
         <v>1313</v>
       </c>
       <c r="D10" s="49">
-        <v>197419.3</v>
+        <v>195674.89999999994</v>
       </c>
       <c r="E10" t="s">
         <v>1334</v>
@@ -6257,14 +6257,16 @@
         <v>56</v>
       </c>
       <c r="B11" s="68" t="s">
-        <v>1360</v>
+        <v>1358</v>
       </c>
       <c r="C11" s="68" t="s">
-        <v>1313</v>
-      </c>
-      <c r="D11" s="69"/>
+        <v>1358</v>
+      </c>
+      <c r="D11" s="69">
+        <v>191319.80000000002</v>
+      </c>
       <c r="E11" s="68" t="s">
-        <v>1361</v>
+        <v>1359</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -6272,16 +6274,16 @@
         <v>60</v>
       </c>
       <c r="B12" t="s">
-        <v>1358</v>
+        <v>1356</v>
       </c>
       <c r="C12" t="s">
-        <v>1358</v>
+        <v>1356</v>
       </c>
       <c r="D12" s="49">
-        <v>3513056.16</v>
+        <v>3706435.56</v>
       </c>
       <c r="E12" t="s">
-        <v>1335</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -6289,16 +6291,16 @@
         <v>60</v>
       </c>
       <c r="B13" t="s">
-        <v>1359</v>
+        <v>1357</v>
       </c>
       <c r="C13" t="s">
-        <v>1359</v>
+        <v>1357</v>
       </c>
       <c r="D13" s="49">
         <v>4383866.2385710711</v>
       </c>
       <c r="E13" t="s">
-        <v>1336</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -6306,16 +6308,16 @@
         <v>64</v>
       </c>
       <c r="B14" s="68" t="s">
-        <v>1381</v>
+        <v>1379</v>
       </c>
       <c r="C14" s="68" t="s">
-        <v>1338</v>
+        <v>1336</v>
       </c>
       <c r="D14" s="69">
         <v>99153.400000000009</v>
       </c>
       <c r="E14" s="68" t="s">
-        <v>1338</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -6323,16 +6325,16 @@
         <v>64</v>
       </c>
       <c r="B15" s="68" t="s">
-        <v>1382</v>
+        <v>1380</v>
       </c>
       <c r="C15" s="68" t="s">
-        <v>1339</v>
+        <v>1337</v>
       </c>
       <c r="D15" s="69">
         <v>73679.429999999993</v>
       </c>
       <c r="E15" s="68" t="s">
-        <v>1339</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -6340,17 +6342,17 @@
         <v>64</v>
       </c>
       <c r="B16" s="68" t="s">
-        <v>1383</v>
+        <v>1381</v>
       </c>
       <c r="C16" s="68" t="s">
-        <v>1362</v>
+        <v>1360</v>
       </c>
       <c r="D16" s="69">
         <f>SUM(D14:D15)</f>
         <v>172832.83000000002</v>
       </c>
       <c r="E16" s="68" t="s">
-        <v>1362</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -6358,10 +6360,10 @@
         <v>68</v>
       </c>
       <c r="B17" t="s">
-        <v>1365</v>
+        <v>1363</v>
       </c>
       <c r="C17" t="s">
-        <v>1363</v>
+        <v>1361</v>
       </c>
       <c r="D17" s="49">
         <v>0</v>
@@ -6375,10 +6377,10 @@
         <v>68</v>
       </c>
       <c r="B18" t="s">
-        <v>1366</v>
+        <v>1364</v>
       </c>
       <c r="C18" t="s">
-        <v>1363</v>
+        <v>1361</v>
       </c>
       <c r="D18" s="49">
         <v>0</v>
@@ -6392,10 +6394,10 @@
         <v>68</v>
       </c>
       <c r="B19" t="s">
-        <v>1367</v>
+        <v>1365</v>
       </c>
       <c r="C19" t="s">
-        <v>1363</v>
+        <v>1361</v>
       </c>
       <c r="D19" s="49">
         <v>0</v>
@@ -6409,10 +6411,10 @@
         <v>68</v>
       </c>
       <c r="B20" t="s">
-        <v>1368</v>
+        <v>1366</v>
       </c>
       <c r="C20" t="s">
-        <v>1363</v>
+        <v>1361</v>
       </c>
       <c r="D20" s="49">
         <f>Sheet1!R18</f>
@@ -6427,10 +6429,10 @@
         <v>68</v>
       </c>
       <c r="B21" t="s">
-        <v>1369</v>
+        <v>1367</v>
       </c>
       <c r="C21" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="D21" s="49">
         <f>SUM(D17:D20)</f>
@@ -6445,10 +6447,10 @@
         <v>71</v>
       </c>
       <c r="B22" t="s">
-        <v>1370</v>
+        <v>1368</v>
       </c>
       <c r="C22" t="s">
-        <v>1364</v>
+        <v>1362</v>
       </c>
       <c r="E22" t="s">
         <v>101</v>
@@ -6459,10 +6461,10 @@
         <v>71</v>
       </c>
       <c r="B23" t="s">
-        <v>1371</v>
+        <v>1369</v>
       </c>
       <c r="C23" t="s">
-        <v>1364</v>
+        <v>1362</v>
       </c>
       <c r="E23" t="s">
         <v>102</v>
@@ -6473,10 +6475,10 @@
         <v>71</v>
       </c>
       <c r="B24" t="s">
-        <v>1372</v>
+        <v>1370</v>
       </c>
       <c r="C24" t="s">
-        <v>1364</v>
+        <v>1362</v>
       </c>
       <c r="D24" s="49">
         <f>Sheet1!R15</f>
@@ -6491,10 +6493,10 @@
         <v>71</v>
       </c>
       <c r="B25" t="s">
-        <v>1373</v>
+        <v>1371</v>
       </c>
       <c r="C25" t="s">
-        <v>1364</v>
+        <v>1362</v>
       </c>
       <c r="D25" s="49">
         <f>Sheet1!R16</f>
@@ -6509,7 +6511,7 @@
         <v>71</v>
       </c>
       <c r="B26" t="s">
-        <v>1374</v>
+        <v>1372</v>
       </c>
       <c r="C26" t="s">
         <v>106</v>
@@ -6928,42 +6930,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="17.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="83" t="s">
+      <c r="A1" s="87" t="s">
+        <v>1339</v>
+      </c>
+      <c r="B1" s="88"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="87" t="s">
+        <v>1340</v>
+      </c>
+      <c r="F1" s="88"/>
+      <c r="G1" s="89"/>
+    </row>
+    <row r="2" spans="1:7" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="52" t="s">
         <v>1341</v>
       </c>
-      <c r="B1" s="84"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="83" t="s">
+      <c r="B2" s="53" t="s">
         <v>1342</v>
       </c>
-      <c r="F1" s="84"/>
-      <c r="G1" s="85"/>
-    </row>
-    <row r="2" spans="1:7" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="52" t="s">
+      <c r="C2" s="54" t="s">
         <v>1343</v>
-      </c>
-      <c r="B2" s="53" t="s">
-        <v>1344</v>
-      </c>
-      <c r="C2" s="54" t="s">
-        <v>1345</v>
       </c>
       <c r="D2" s="51"/>
       <c r="E2" s="55" t="s">
+        <v>1341</v>
+      </c>
+      <c r="F2" s="53" t="s">
+        <v>1342</v>
+      </c>
+      <c r="G2" s="54" t="s">
         <v>1343</v>
-      </c>
-      <c r="F2" s="53" t="s">
-        <v>1344</v>
-      </c>
-      <c r="G2" s="54" t="s">
-        <v>1345</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="52" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B3" s="53">
         <v>63</v>
@@ -6973,7 +6975,7 @@
       </c>
       <c r="D3" s="51"/>
       <c r="E3" s="55" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="F3" s="53">
         <v>55</v>
@@ -6984,7 +6986,7 @@
     </row>
     <row r="4" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="52" t="s">
-        <v>1348</v>
+        <v>1346</v>
       </c>
       <c r="B4" s="53">
         <v>24</v>
@@ -6994,7 +6996,7 @@
       </c>
       <c r="D4" s="51"/>
       <c r="E4" s="55" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="F4" s="53">
         <v>32</v>
@@ -7005,7 +7007,7 @@
     </row>
     <row r="5" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="52" t="s">
-        <v>1350</v>
+        <v>1348</v>
       </c>
       <c r="B5" s="53">
         <v>4</v>
@@ -7015,7 +7017,7 @@
       </c>
       <c r="D5" s="51"/>
       <c r="E5" s="55" t="s">
-        <v>1351</v>
+        <v>1349</v>
       </c>
       <c r="F5" s="53">
         <v>0</v>
@@ -7026,7 +7028,7 @@
     </row>
     <row r="6" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="56" t="s">
-        <v>1352</v>
+        <v>1350</v>
       </c>
       <c r="B6" s="57">
         <v>0</v>
@@ -7036,7 +7038,7 @@
       </c>
       <c r="D6" s="51"/>
       <c r="E6" s="59" t="s">
-        <v>1352</v>
+        <v>1350</v>
       </c>
       <c r="F6" s="57">
         <v>0</v>
@@ -7047,27 +7049,27 @@
     </row>
     <row r="7" spans="1:7" ht="16.5" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="22" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="81" t="s">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="85" t="s">
         <v>149</v>
       </c>
-      <c r="B22" s="82"/>
+      <c r="B22" s="86"/>
       <c r="C22" s="60"/>
       <c r="D22" s="61"/>
-      <c r="E22" s="81" t="s">
+      <c r="E22" s="85" t="s">
         <v>150</v>
       </c>
-      <c r="F22" s="82"/>
+      <c r="F22" s="86"/>
       <c r="G22" s="62" t="s">
-        <v>1353</v>
+        <v>1351</v>
       </c>
       <c r="H22" s="61"/>
-      <c r="I22" s="81" t="s">
+      <c r="I22" s="85" t="s">
         <v>151</v>
       </c>
-      <c r="J22" s="82"/>
-      <c r="K22" s="86" t="s">
-        <v>1353</v>
+      <c r="J22" s="86"/>
+      <c r="K22" s="81" t="s">
+        <v>1351</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
@@ -7095,7 +7097,7 @@
       <c r="J23" s="64" t="s">
         <v>153</v>
       </c>
-      <c r="K23" s="87" t="s">
+      <c r="K23" s="82" t="s">
         <v>154</v>
       </c>
     </row>
@@ -7104,7 +7106,7 @@
         <v>883</v>
       </c>
       <c r="B24" s="71" t="s">
-        <v>1356</v>
+        <v>1354</v>
       </c>
       <c r="C24" s="60"/>
       <c r="D24" s="65"/>
@@ -7112,9 +7114,9 @@
         <v>931</v>
       </c>
       <c r="F24" s="71" t="s">
-        <v>1390</v>
-      </c>
-      <c r="G24" s="88" t="s">
+        <v>1388</v>
+      </c>
+      <c r="G24" s="83" t="s">
         <v>157</v>
       </c>
       <c r="H24" s="65"/>
@@ -7122,7 +7124,7 @@
         <v>903</v>
       </c>
       <c r="J24" s="74" t="s">
-        <v>1389</v>
+        <v>1387</v>
       </c>
       <c r="K24" s="77" t="s">
         <v>157</v>
@@ -7133,22 +7135,22 @@
         <v>863</v>
       </c>
       <c r="B25" s="67" t="s">
-        <v>1389</v>
+        <v>1387</v>
       </c>
       <c r="E25" s="70" t="s">
         <v>895</v>
       </c>
       <c r="F25" s="71" t="s">
-        <v>1356</v>
-      </c>
-      <c r="G25" s="88" t="s">
+        <v>1354</v>
+      </c>
+      <c r="G25" s="83" t="s">
         <v>160</v>
       </c>
       <c r="I25" s="73" t="s">
         <v>923</v>
       </c>
       <c r="J25" s="74" t="s">
-        <v>1390</v>
+        <v>1388</v>
       </c>
       <c r="K25" s="77" t="s">
         <v>157</v>
@@ -7161,16 +7163,16 @@
         <v>887</v>
       </c>
       <c r="F26" s="67" t="s">
-        <v>1356</v>
-      </c>
-      <c r="G26" s="89" t="s">
+        <v>1354</v>
+      </c>
+      <c r="G26" s="84" t="s">
         <v>157</v>
       </c>
       <c r="I26" s="73" t="s">
         <v>967</v>
       </c>
       <c r="J26" s="74" t="s">
-        <v>1390</v>
+        <v>1388</v>
       </c>
       <c r="K26" s="77" t="s">
         <v>157</v>
@@ -7183,7 +7185,7 @@
         <v>971</v>
       </c>
       <c r="J27" s="74" t="s">
-        <v>1356</v>
+        <v>1354</v>
       </c>
       <c r="K27" s="77" t="s">
         <v>157</v>
@@ -7196,7 +7198,7 @@
         <v>155</v>
       </c>
       <c r="J28" s="74" t="s">
-        <v>1391</v>
+        <v>1389</v>
       </c>
       <c r="K28" s="77" t="s">
         <v>157</v>
@@ -7207,7 +7209,7 @@
         <v>811</v>
       </c>
       <c r="J29" s="76" t="s">
-        <v>1390</v>
+        <v>1388</v>
       </c>
       <c r="K29" s="78" t="s">
         <v>157</v>
@@ -35282,7 +35284,7 @@
         <v>160</v>
       </c>
       <c r="T142" s="36" t="s">
-        <v>1378</v>
+        <v>1376</v>
       </c>
       <c r="U142" s="34">
         <v>779</v>
@@ -37039,10 +37041,10 @@
         <v>46215</v>
       </c>
       <c r="O152" s="36" t="s">
-        <v>1379</v>
+        <v>1377</v>
       </c>
       <c r="P152" s="41" t="s">
-        <v>1380</v>
+        <v>1378</v>
       </c>
       <c r="Q152" s="36" t="s">
         <v>258</v>
@@ -37052,7 +37054,7 @@
       </c>
       <c r="S152" s="36"/>
       <c r="T152" s="36" t="s">
-        <v>1378</v>
+        <v>1376</v>
       </c>
       <c r="U152" s="34">
         <v>779</v>
@@ -37199,7 +37201,7 @@
         <v>157</v>
       </c>
       <c r="T153" s="36" t="s">
-        <v>1378</v>
+        <v>1376</v>
       </c>
       <c r="U153" s="34">
         <v>779</v>
@@ -37341,10 +37343,10 @@
         <v>46214</v>
       </c>
       <c r="O154" s="36" t="s">
-        <v>1379</v>
+        <v>1377</v>
       </c>
       <c r="P154" s="41" t="s">
-        <v>1380</v>
+        <v>1378</v>
       </c>
       <c r="Q154" s="36" t="s">
         <v>258</v>
@@ -37356,7 +37358,7 @@
         <v>863</v>
       </c>
       <c r="T154" s="36" t="s">
-        <v>1378</v>
+        <v>1376</v>
       </c>
       <c r="U154" s="34">
         <v>779</v>
@@ -38175,7 +38177,7 @@
       </c>
       <c r="S159" s="36"/>
       <c r="T159" s="36" t="s">
-        <v>1384</v>
+        <v>1382</v>
       </c>
       <c r="U159" s="34">
         <v>779</v>
@@ -38307,10 +38309,10 @@
         <v>46212</v>
       </c>
       <c r="O160" s="36" t="s">
-        <v>1379</v>
+        <v>1377</v>
       </c>
       <c r="P160" s="41" t="s">
-        <v>1380</v>
+        <v>1378</v>
       </c>
       <c r="Q160" s="36" t="s">
         <v>258</v>
@@ -38322,7 +38324,7 @@
         <v>157</v>
       </c>
       <c r="T160" s="36" t="s">
-        <v>1378</v>
+        <v>1376</v>
       </c>
       <c r="U160" s="34">
         <v>779</v>
@@ -38601,10 +38603,10 @@
         <v>46214</v>
       </c>
       <c r="O162" s="36" t="s">
-        <v>1379</v>
+        <v>1377</v>
       </c>
       <c r="P162" s="41" t="s">
-        <v>1380</v>
+        <v>1378</v>
       </c>
       <c r="Q162" s="36" t="s">
         <v>258</v>
@@ -38616,7 +38618,7 @@
         <v>160</v>
       </c>
       <c r="T162" s="36" t="s">
-        <v>1378</v>
+        <v>1376</v>
       </c>
       <c r="U162" s="34">
         <v>779</v>
@@ -39441,7 +39443,7 @@
         <v>157</v>
       </c>
       <c r="T167" s="36" t="s">
-        <v>1378</v>
+        <v>1376</v>
       </c>
       <c r="U167" s="34">
         <v>779</v>
@@ -39774,10 +39776,10 @@
         <v>46208</v>
       </c>
       <c r="O169" s="36" t="s">
-        <v>1379</v>
+        <v>1377</v>
       </c>
       <c r="P169" s="41" t="s">
-        <v>1380</v>
+        <v>1378</v>
       </c>
       <c r="Q169" s="36" t="s">
         <v>258</v>
@@ -40072,10 +40074,10 @@
         <v>46212</v>
       </c>
       <c r="O171" s="36" t="s">
-        <v>1379</v>
+        <v>1377</v>
       </c>
       <c r="P171" s="41" t="s">
-        <v>1380</v>
+        <v>1378</v>
       </c>
       <c r="Q171" s="36" t="s">
         <v>258</v>
@@ -40087,7 +40089,7 @@
         <v>157</v>
       </c>
       <c r="T171" s="36" t="s">
-        <v>1378</v>
+        <v>1376</v>
       </c>
       <c r="U171" s="34">
         <v>779</v>
@@ -41019,10 +41021,10 @@
         <v>46209</v>
       </c>
       <c r="O176" s="36" t="s">
-        <v>1379</v>
+        <v>1377</v>
       </c>
       <c r="P176" s="41" t="s">
-        <v>1380</v>
+        <v>1378</v>
       </c>
       <c r="Q176" s="36" t="s">
         <v>258</v>
@@ -41034,7 +41036,7 @@
         <v>160</v>
       </c>
       <c r="T176" s="36" t="s">
-        <v>1378</v>
+        <v>1376</v>
       </c>
       <c r="U176" s="34">
         <v>779</v>
@@ -41869,7 +41871,7 @@
         <v>157</v>
       </c>
       <c r="T181" s="36" t="s">
-        <v>1378</v>
+        <v>1376</v>
       </c>
       <c r="U181" s="34">
         <v>779</v>
@@ -47304,7 +47306,7 @@
         <v>1107</v>
       </c>
       <c r="T214" s="36" t="s">
-        <v>1378</v>
+        <v>1376</v>
       </c>
       <c r="U214" s="34">
         <v>0</v>
@@ -54020,7 +54022,7 @@
     </row>
     <row r="261" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A261" s="36" t="s">
-        <v>1385</v>
+        <v>1383</v>
       </c>
       <c r="B261" s="36" t="s">
         <v>1280</v>
@@ -54071,7 +54073,7 @@
         <v>1107</v>
       </c>
       <c r="T261" s="36" t="s">
-        <v>1378</v>
+        <v>1376</v>
       </c>
       <c r="U261" s="34">
         <v>0</v>
@@ -54161,7 +54163,7 @@
     </row>
     <row r="262" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A262" s="36" t="s">
-        <v>1386</v>
+        <v>1384</v>
       </c>
       <c r="B262" s="36" t="s">
         <v>1283</v>
@@ -54212,7 +54214,7 @@
         <v>1107</v>
       </c>
       <c r="T262" s="36" t="s">
-        <v>1378</v>
+        <v>1376</v>
       </c>
       <c r="U262" s="34">
         <v>0</v>
@@ -72132,7 +72134,7 @@
   <sheetData>
     <row r="2" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B2" s="79" t="s">
-        <v>1337</v>
+        <v>1335</v>
       </c>
       <c r="C2" t="s">
         <v>1289</v>
@@ -72328,10 +72330,10 @@
         <v>1306</v>
       </c>
       <c r="S7">
-        <v>1566141</v>
+        <v>1605916</v>
       </c>
       <c r="T7">
-        <v>1566141</v>
+        <v>1605916</v>
       </c>
     </row>
     <row r="8" spans="2:20" x14ac:dyDescent="0.25">
@@ -72378,10 +72380,10 @@
         <v>1308</v>
       </c>
       <c r="S8">
-        <v>1566141</v>
+        <v>1605916</v>
       </c>
       <c r="T8">
-        <v>1566141</v>
+        <v>1605916</v>
       </c>
     </row>
     <row r="9" spans="2:20" x14ac:dyDescent="0.25">
@@ -72500,7 +72502,7 @@
     </row>
     <row r="12" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B12" s="79" t="s">
-        <v>1357</v>
+        <v>1355</v>
       </c>
       <c r="C12" t="s">
         <v>1289</v>
@@ -72579,7 +72581,7 @@
         <v>1300</v>
       </c>
       <c r="Q14" t="s">
-        <v>1387</v>
+        <v>1385</v>
       </c>
       <c r="R14">
         <v>67811.759999999966</v>
@@ -72711,7 +72713,7 @@
         <v>69424.33</v>
       </c>
       <c r="Q17" t="s">
-        <v>1388</v>
+        <v>1386</v>
       </c>
       <c r="R17">
         <v>64299.000000000036</v>
@@ -72775,40 +72777,40 @@
         <v>1308</v>
       </c>
       <c r="C19">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="D19">
-        <v>194309</v>
+        <v>304683</v>
       </c>
       <c r="E19">
-        <v>58730.000000000029</v>
+        <v>93424.46000000005</v>
       </c>
       <c r="F19">
-        <v>893</v>
+        <v>933</v>
       </c>
       <c r="G19">
-        <v>1803914.4</v>
+        <v>1839043.4</v>
       </c>
       <c r="H19">
-        <v>106536.12000000029</v>
+        <v>114447.4200000003</v>
       </c>
       <c r="I19">
-        <v>660</v>
+        <v>615</v>
       </c>
       <c r="J19">
-        <v>1867434</v>
+        <v>1746915</v>
       </c>
       <c r="K19">
-        <v>1867434</v>
+        <v>1746915</v>
       </c>
       <c r="L19">
-        <v>1631</v>
+        <v>1640</v>
       </c>
       <c r="M19">
-        <v>3865657.4</v>
+        <v>3890641.4</v>
       </c>
       <c r="N19">
-        <v>2032700.1200000003</v>
+        <v>1954786.8800000001</v>
       </c>
       <c r="Q19" t="s">
         <v>1304</v>
@@ -72817,10 +72819,10 @@
         <v>498268.12000000005</v>
       </c>
       <c r="S19">
-        <v>1798403.96</v>
+        <v>1838178.96</v>
       </c>
       <c r="T19">
-        <v>2296672.0799999996</v>
+        <v>2336447.0799999996</v>
       </c>
     </row>
     <row r="20" spans="2:20" x14ac:dyDescent="0.25">
@@ -72828,40 +72830,40 @@
         <v>1304</v>
       </c>
       <c r="C20">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="D20">
-        <v>452159</v>
+        <v>562533</v>
       </c>
       <c r="E20" s="79">
-        <v>127353.50000000003</v>
+        <v>162047.95999999996</v>
       </c>
       <c r="F20">
-        <v>17860</v>
+        <v>17900</v>
       </c>
       <c r="G20">
-        <v>43561093.870000236</v>
+        <v>43596222.870000236</v>
       </c>
       <c r="H20">
-        <v>150584.22000000023</v>
+        <v>158495.52000000028</v>
       </c>
       <c r="I20">
-        <v>709</v>
+        <v>664</v>
       </c>
       <c r="J20">
-        <v>2117823</v>
+        <v>1997304</v>
       </c>
       <c r="K20" s="79">
-        <v>2117823</v>
+        <v>1997304</v>
       </c>
       <c r="L20">
-        <v>18670</v>
+        <v>18679</v>
       </c>
       <c r="M20">
-        <v>46131075.870000027</v>
+        <v>46156059.870000027</v>
       </c>
       <c r="N20" s="79">
-        <v>2395760.7200000002</v>
+        <v>2317847.48</v>
       </c>
     </row>
     <row r="25" spans="2:20" x14ac:dyDescent="0.25">
@@ -72921,7 +72923,7 @@
         <v>2025</v>
       </c>
       <c r="R32">
-        <f t="shared" ref="R31:R33" si="0">R12</f>
+        <f t="shared" ref="R32:R33" si="0">R12</f>
         <v>132175.70000000001</v>
       </c>
     </row>

</xml_diff>

<commit_message>
UI: Move QC Overview, Operation Error, and Improvement Plan cards to the bottom
</commit_message>
<xml_diff>
--- a/Dashboard_Template_30_Slides_Final.xlsx
+++ b/Dashboard_Template_30_Slides_Final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\0_Dashboad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE982FBA-EA34-410F-989E-CCC866D46D27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B255C16-776D-4088-91A0-6203D90D83C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="813" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="813" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Part 1 - Overview" sheetId="1" r:id="rId1"/>
@@ -5107,12 +5107,6 @@
     <xf numFmtId="0" fontId="20" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -5120,6 +5114,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6930,17 +6930,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="17.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="87" t="s">
+      <c r="A1" s="85" t="s">
         <v>1338</v>
       </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="89"/>
+      <c r="B1" s="86"/>
+      <c r="C1" s="87"/>
       <c r="D1" s="51"/>
-      <c r="E1" s="87" t="s">
+      <c r="E1" s="85" t="s">
         <v>1339</v>
       </c>
-      <c r="F1" s="88"/>
-      <c r="G1" s="89"/>
+      <c r="F1" s="86"/>
+      <c r="G1" s="87"/>
     </row>
     <row r="2" spans="1:7" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="52" t="s">
@@ -6968,20 +6968,20 @@
         <v>1343</v>
       </c>
       <c r="B3" s="53">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="C3" s="54">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="D3" s="51"/>
       <c r="E3" s="55" t="s">
         <v>1344</v>
       </c>
       <c r="F3" s="53">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="G3" s="54">
-        <v>3</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -6989,20 +6989,20 @@
         <v>1345</v>
       </c>
       <c r="B4" s="53">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C4" s="54">
-        <v>7</v>
+        <v>6.9</v>
       </c>
       <c r="D4" s="51"/>
       <c r="E4" s="55" t="s">
         <v>1346</v>
       </c>
       <c r="F4" s="53">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G4" s="54">
-        <v>10</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -7010,20 +7010,20 @@
         <v>1347</v>
       </c>
       <c r="B5" s="53">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C5" s="54">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D5" s="51"/>
       <c r="E5" s="55" t="s">
         <v>1348</v>
       </c>
       <c r="F5" s="53">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G5" s="54">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -7050,24 +7050,24 @@
     <row r="7" spans="1:7" ht="16.5" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="85" t="s">
+      <c r="A22" s="88" t="s">
         <v>148</v>
       </c>
-      <c r="B22" s="86"/>
+      <c r="B22" s="89"/>
       <c r="C22" s="60"/>
       <c r="D22" s="61"/>
-      <c r="E22" s="85" t="s">
+      <c r="E22" s="88" t="s">
         <v>149</v>
       </c>
-      <c r="F22" s="86"/>
+      <c r="F22" s="89"/>
       <c r="G22" s="62" t="s">
         <v>1350</v>
       </c>
       <c r="H22" s="61"/>
-      <c r="I22" s="85" t="s">
+      <c r="I22" s="88" t="s">
         <v>150</v>
       </c>
-      <c r="J22" s="86"/>
+      <c r="J22" s="89"/>
       <c r="K22" s="81" t="s">
         <v>1350</v>
       </c>
@@ -7216,10 +7216,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="3">
     <mergeCell ref="I22:J22"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="E1:G1"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="E22:F22"/>
   </mergeCells>

</xml_diff>

<commit_message>
Move Install On-Process card to right of Site Completion
</commit_message>
<xml_diff>
--- a/Dashboard_Template_30_Slides_Final.xlsx
+++ b/Dashboard_Template_30_Slides_Final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\0_Dashboad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B255C16-776D-4088-91A0-6203D90D83C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1D699E9-75AB-4CA4-A959-2E74407C4938}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="813" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="813" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Part 1 - Overview" sheetId="1" r:id="rId1"/>
@@ -200,7 +200,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5261" uniqueCount="1392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5256" uniqueCount="1392">
   <si>
     <t>Slide No</t>
   </si>
@@ -5904,13 +5904,13 @@
         <v>1373</v>
       </c>
       <c r="D3">
-        <v>247932</v>
+        <v>234856</v>
       </c>
       <c r="E3" t="s">
         <v>17</v>
       </c>
       <c r="F3">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G3" t="s">
         <v>1372</v>
@@ -7518,11 +7518,11 @@
       </c>
       <c r="L2" s="10">
         <f t="shared" si="0"/>
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M2" s="10">
         <f t="shared" si="0"/>
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="N2" s="10">
         <f t="shared" si="0"/>
@@ -7530,19 +7530,19 @@
       </c>
       <c r="O2" s="10">
         <f t="shared" si="0"/>
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P2" s="10">
         <f t="shared" si="0"/>
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="Q2" s="10">
         <f t="shared" si="0"/>
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="R2" s="10">
         <f t="shared" si="0"/>
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="S2" s="10">
         <f t="shared" si="0"/>
@@ -7550,7 +7550,7 @@
       </c>
       <c r="T2" s="10">
         <f t="shared" si="0"/>
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="U2" s="12">
         <f>SUBTOTAL(9,U4:U263)</f>
@@ -28014,7 +28014,7 @@
         <v>605</v>
       </c>
       <c r="S105" s="36" t="s">
-        <v>45</v>
+        <v>605</v>
       </c>
       <c r="T105" s="36"/>
       <c r="U105" s="34">
@@ -37029,31 +37029,17 @@
       <c r="K152" s="36" t="s">
         <v>236</v>
       </c>
-      <c r="L152" s="40">
-        <v>46215</v>
-      </c>
-      <c r="M152" s="40">
-        <v>46215</v>
-      </c>
+      <c r="L152" s="40"/>
+      <c r="M152" s="40"/>
       <c r="N152" s="41">
-        <v>46215</v>
-      </c>
-      <c r="O152" s="36" t="s">
-        <v>1375</v>
-      </c>
-      <c r="P152" s="41" t="s">
-        <v>1376</v>
-      </c>
-      <c r="Q152" s="36" t="s">
-        <v>257</v>
-      </c>
-      <c r="R152" s="36" t="s">
-        <v>45</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O152" s="36"/>
+      <c r="P152" s="41"/>
+      <c r="Q152" s="36"/>
+      <c r="R152" s="36"/>
       <c r="S152" s="36"/>
-      <c r="T152" s="36" t="s">
-        <v>1374</v>
-      </c>
+      <c r="T152" s="36"/>
       <c r="U152" s="34">
         <v>779</v>
       </c>
@@ -37114,7 +37100,7 @@
       <c r="BD152" s="36"/>
       <c r="BE152" s="36"/>
       <c r="BF152" s="36" t="s">
-        <v>243</v>
+        <v>802</v>
       </c>
       <c r="BG152" s="36" t="s">
         <v>111</v>

</xml_diff>